<commit_message>
xlsx ouput issues fixed
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_appliance.xlsx
+++ b/Ground Truth/ground_truth_appliance.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R295"/>
+  <dimension ref="A1:R289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18726,50 +18726,50 @@
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>It's around 8 in the morning and I need to run the dishwasher. When should I start it?</t>
+          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Levittown, PA</t>
+          <t>Pottstown, PA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>dishwasher</t>
+          <t>washing_machine</t>
         </is>
       </c>
       <c r="F278" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H278" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I278" t="n">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>8:00 AM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="K278" t="n">
-        <v>10</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="L278" t="n">
-        <v>8.119999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M278" t="n">
         <v>10</v>
@@ -18778,64 +18778,64 @@
         <v>10</v>
       </c>
       <c r="O278" t="n">
-        <v>9.341999999999999</v>
+        <v>9.714</v>
       </c>
       <c r="P278" t="n">
         <v>1</v>
       </c>
       <c r="Q278" t="n">
-        <v>0</v>
+        <v>0.096</v>
       </c>
       <c r="R278" t="n">
-        <v>0.885</v>
+        <v>0.312</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>It's around 8 in the morning and I need to run the dishwasher. When should I start it?</t>
+          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Levittown, PA</t>
+          <t>Pottstown, PA</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>dishwasher</t>
+          <t>washing_machine</t>
         </is>
       </c>
       <c r="F279" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H279" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I279" t="n">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>9:00 PM</t>
         </is>
       </c>
       <c r="K279" t="n">
-        <v>10</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="L279" t="n">
-        <v>8.119999999999999</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M279" t="n">
         <v>7.43</v>
@@ -18844,130 +18844,130 @@
         <v>6.21</v>
       </c>
       <c r="O279" t="n">
-        <v>8.259499999999999</v>
+        <v>8.8325</v>
       </c>
       <c r="P279" t="n">
         <v>2</v>
       </c>
       <c r="Q279" t="n">
-        <v>0</v>
+        <v>0.0228</v>
       </c>
       <c r="R279" t="n">
-        <v>0.885</v>
+        <v>0.312</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>It's around 8 in the morning and I need to run the dishwasher. When should I start it?</t>
+          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Levittown, PA</t>
+          <t>Pottstown, PA</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>dishwasher</t>
+          <t>washing_machine</t>
         </is>
       </c>
       <c r="F280" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H280" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I280" t="n">
-        <v>0.85</v>
+        <v>0.3</v>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>11:00 PM</t>
+          <t>6:00 AM</t>
         </is>
       </c>
       <c r="K280" t="n">
-        <v>10</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="L280" t="n">
-        <v>8.279999999999999</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="M280" t="n">
-        <v>6.29</v>
+        <v>4.71</v>
       </c>
       <c r="N280" t="n">
-        <v>3.63</v>
+        <v>4.78</v>
       </c>
       <c r="O280" t="n">
-        <v>7.7005</v>
+        <v>8.095000000000001</v>
       </c>
       <c r="P280" t="n">
         <v>3</v>
       </c>
       <c r="Q280" t="n">
-        <v>0</v>
+        <v>0.0228</v>
       </c>
       <c r="R280" t="n">
-        <v>0.83</v>
+        <v>0.293</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
+          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Pottstown, PA</t>
+          <t>Phoenixville, PA</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>washing_machine</t>
+          <t>dryer</t>
         </is>
       </c>
       <c r="F281" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Townhouse</t>
         </is>
       </c>
       <c r="H281" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I281" t="n">
-        <v>0.3</v>
+        <v>2.8</v>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="K281" t="n">
-        <v>9.279999999999999</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="L281" t="n">
-        <v>9.800000000000001</v>
+        <v>2.14</v>
       </c>
       <c r="M281" t="n">
         <v>10</v>
@@ -18976,166 +18976,166 @@
         <v>10</v>
       </c>
       <c r="O281" t="n">
-        <v>9.714</v>
+        <v>6.715</v>
       </c>
       <c r="P281" t="n">
         <v>1</v>
       </c>
       <c r="Q281" t="n">
-        <v>0.096</v>
+        <v>0.2128</v>
       </c>
       <c r="R281" t="n">
-        <v>0.312</v>
+        <v>2.915</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
+          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Pottstown, PA</t>
+          <t>Phoenixville, PA</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>washing_machine</t>
+          <t>dryer</t>
         </is>
       </c>
       <c r="F282" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Townhouse</t>
         </is>
       </c>
       <c r="H282" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I282" t="n">
-        <v>0.3</v>
+        <v>2.8</v>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>9:00 PM</t>
+          <t>11:00 PM</t>
         </is>
       </c>
       <c r="K282" t="n">
-        <v>9.949999999999999</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="L282" t="n">
-        <v>9.800000000000001</v>
+        <v>2.68</v>
       </c>
       <c r="M282" t="n">
-        <v>7.43</v>
+        <v>6.2</v>
       </c>
       <c r="N282" t="n">
         <v>6.21</v>
       </c>
       <c r="O282" t="n">
-        <v>8.8325</v>
+        <v>5.5755</v>
       </c>
       <c r="P282" t="n">
         <v>2</v>
       </c>
       <c r="Q282" t="n">
-        <v>0.0228</v>
+        <v>0.2128</v>
       </c>
       <c r="R282" t="n">
-        <v>0.312</v>
+        <v>2.733</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
+          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Pottstown, PA</t>
+          <t>Phoenixville, PA</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>washing_machine</t>
+          <t>dryer</t>
         </is>
       </c>
       <c r="F283" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Townhouse</t>
         </is>
       </c>
       <c r="H283" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I283" t="n">
-        <v>0.3</v>
+        <v>2.8</v>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>6:00 AM</t>
+          <t>8:00 AM</t>
         </is>
       </c>
       <c r="K283" t="n">
-        <v>9.949999999999999</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="L283" t="n">
-        <v>9.859999999999999</v>
+        <v>2.14</v>
       </c>
       <c r="M283" t="n">
-        <v>4.71</v>
+        <v>5.53</v>
       </c>
       <c r="N283" t="n">
-        <v>4.78</v>
+        <v>3.93</v>
       </c>
       <c r="O283" t="n">
-        <v>8.095000000000001</v>
+        <v>4.910500000000001</v>
       </c>
       <c r="P283" t="n">
         <v>3</v>
       </c>
       <c r="Q283" t="n">
-        <v>0.0228</v>
+        <v>0.2128</v>
       </c>
       <c r="R283" t="n">
-        <v>0.293</v>
+        <v>2.915</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Phoenixville, PA</t>
+          <t>McKeesport, PA</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>155</v>
+        <v>220</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -19143,7 +19143,7 @@
         </is>
       </c>
       <c r="F284" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G284" t="inlineStr">
         <is>
@@ -19151,21 +19151,21 @@
         </is>
       </c>
       <c r="H284" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I284" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="K284" t="n">
-        <v>8.220000000000001</v>
+        <v>6.91</v>
       </c>
       <c r="L284" t="n">
-        <v>2.14</v>
+        <v>2.76</v>
       </c>
       <c r="M284" t="n">
         <v>10</v>
@@ -19174,34 +19174,34 @@
         <v>10</v>
       </c>
       <c r="O284" t="n">
-        <v>6.715</v>
+        <v>6.539</v>
       </c>
       <c r="P284" t="n">
         <v>1</v>
       </c>
       <c r="Q284" t="n">
-        <v>0.2128</v>
+        <v>0.3575</v>
       </c>
       <c r="R284" t="n">
-        <v>2.915</v>
+        <v>2.707</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Phoenixville, PA</t>
+          <t>McKeesport, PA</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>155</v>
+        <v>220</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -19209,7 +19209,7 @@
         </is>
       </c>
       <c r="F285" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G285" t="inlineStr">
         <is>
@@ -19217,57 +19217,57 @@
         </is>
       </c>
       <c r="H285" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I285" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>11:00 PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="K285" t="n">
-        <v>8.220000000000001</v>
+        <v>6.91</v>
       </c>
       <c r="L285" t="n">
-        <v>2.68</v>
+        <v>2.76</v>
       </c>
       <c r="M285" t="n">
-        <v>6.2</v>
+        <v>7.29</v>
       </c>
       <c r="N285" t="n">
-        <v>6.21</v>
+        <v>6.04</v>
       </c>
       <c r="O285" t="n">
-        <v>5.5755</v>
+        <v>5.403</v>
       </c>
       <c r="P285" t="n">
         <v>2</v>
       </c>
       <c r="Q285" t="n">
-        <v>0.2128</v>
+        <v>0.3575</v>
       </c>
       <c r="R285" t="n">
-        <v>2.733</v>
+        <v>2.707</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Phoenixville, PA</t>
+          <t>McKeesport, PA</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>155</v>
+        <v>220</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -19275,7 +19275,7 @@
         </is>
       </c>
       <c r="F286" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G286" t="inlineStr">
         <is>
@@ -19283,57 +19283,57 @@
         </is>
       </c>
       <c r="H286" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I286" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>8:00 AM</t>
+          <t>10:00 PM</t>
         </is>
       </c>
       <c r="K286" t="n">
-        <v>8.220000000000001</v>
+        <v>6.91</v>
       </c>
       <c r="L286" t="n">
-        <v>2.14</v>
+        <v>2.76</v>
       </c>
       <c r="M286" t="n">
-        <v>5.53</v>
+        <v>3.36</v>
       </c>
       <c r="N286" t="n">
-        <v>3.93</v>
+        <v>3.11</v>
       </c>
       <c r="O286" t="n">
-        <v>4.910500000000001</v>
+        <v>4.1775</v>
       </c>
       <c r="P286" t="n">
         <v>3</v>
       </c>
       <c r="Q286" t="n">
-        <v>0.2128</v>
+        <v>0.3575</v>
       </c>
       <c r="R286" t="n">
-        <v>2.915</v>
+        <v>2.707</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>It's around 11 in the morning and I need to run the dishwasher. When should I start it?</t>
+          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Quakertown, PA</t>
+          <t>Harrisburg, PA</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -19341,29 +19341,29 @@
         </is>
       </c>
       <c r="F287" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H287" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I287" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>11:00 AM</t>
+          <t>6:00 PM</t>
         </is>
       </c>
       <c r="K287" t="n">
-        <v>10</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="L287" t="n">
-        <v>7.35</v>
+        <v>5.51</v>
       </c>
       <c r="M287" t="n">
         <v>10</v>
@@ -19372,34 +19372,34 @@
         <v>10</v>
       </c>
       <c r="O287" t="n">
-        <v>9.0725</v>
+        <v>8.0115</v>
       </c>
       <c r="P287" t="n">
         <v>1</v>
       </c>
       <c r="Q287" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="R287" t="n">
-        <v>1.145</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>It's around 11 in the morning and I need to run the dishwasher. When should I start it?</t>
+          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Quakertown, PA</t>
+          <t>Harrisburg, PA</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -19407,65 +19407,65 @@
         </is>
       </c>
       <c r="F288" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H288" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I288" t="n">
-        <v>1.1</v>
+        <v>1.7</v>
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>9:00 AM</t>
         </is>
       </c>
       <c r="K288" t="n">
-        <v>10</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="L288" t="n">
-        <v>7.35</v>
+        <v>5.51</v>
       </c>
       <c r="M288" t="n">
-        <v>8.23</v>
+        <v>5.21</v>
       </c>
       <c r="N288" t="n">
-        <v>7.15</v>
+        <v>4.64</v>
       </c>
       <c r="O288" t="n">
-        <v>8.291</v>
+        <v>6.249499999999999</v>
       </c>
       <c r="P288" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q288" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="R288" t="n">
-        <v>1.145</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>It's around 11 in the morning and I need to run the dishwasher. When should I start it?</t>
+          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Quakertown, PA</t>
+          <t>Harrisburg, PA</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -19473,442 +19473,46 @@
         </is>
       </c>
       <c r="F289" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Apartment</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H289" t="n">
+        <v>6</v>
+      </c>
+      <c r="I289" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>10:00 PM</t>
+        </is>
+      </c>
+      <c r="K289" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="L289" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="M289" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="N289" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="O289" t="n">
+        <v>6.933999999999999</v>
+      </c>
+      <c r="P289" t="n">
         <v>2</v>
       </c>
-      <c r="I289" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="J289" t="inlineStr">
-        <is>
-          <t>10:00 PM</t>
-        </is>
-      </c>
-      <c r="K289" t="n">
-        <v>10</v>
-      </c>
-      <c r="L289" t="n">
-        <v>7.35</v>
-      </c>
-      <c r="M289" t="n">
-        <v>5.53</v>
-      </c>
-      <c r="N289" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="O289" t="n">
-        <v>7.0835</v>
-      </c>
-      <c r="P289" t="n">
-        <v>3</v>
-      </c>
       <c r="Q289" t="n">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="R289" t="n">
-        <v>1.145</v>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="n">
-        <v>96</v>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
-        </is>
-      </c>
-      <c r="C290" t="inlineStr">
-        <is>
-          <t>McKeesport, PA</t>
-        </is>
-      </c>
-      <c r="D290" t="n">
-        <v>220</v>
-      </c>
-      <c r="E290" t="inlineStr">
-        <is>
-          <t>dryer</t>
-        </is>
-      </c>
-      <c r="F290" t="n">
-        <v>7</v>
-      </c>
-      <c r="G290" t="inlineStr">
-        <is>
-          <t>Townhouse</t>
-        </is>
-      </c>
-      <c r="H290" t="n">
-        <v>4</v>
-      </c>
-      <c r="I290" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="J290" t="inlineStr">
-        <is>
-          <t>2:00 PM</t>
-        </is>
-      </c>
-      <c r="K290" t="n">
-        <v>6.91</v>
-      </c>
-      <c r="L290" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="M290" t="n">
-        <v>10</v>
-      </c>
-      <c r="N290" t="n">
-        <v>10</v>
-      </c>
-      <c r="O290" t="n">
-        <v>6.539</v>
-      </c>
-      <c r="P290" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q290" t="n">
-        <v>0.3575</v>
-      </c>
-      <c r="R290" t="n">
-        <v>2.707</v>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="n">
-        <v>96</v>
-      </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
-        </is>
-      </c>
-      <c r="C291" t="inlineStr">
-        <is>
-          <t>McKeesport, PA</t>
-        </is>
-      </c>
-      <c r="D291" t="n">
-        <v>220</v>
-      </c>
-      <c r="E291" t="inlineStr">
-        <is>
-          <t>dryer</t>
-        </is>
-      </c>
-      <c r="F291" t="n">
-        <v>7</v>
-      </c>
-      <c r="G291" t="inlineStr">
-        <is>
-          <t>Townhouse</t>
-        </is>
-      </c>
-      <c r="H291" t="n">
-        <v>4</v>
-      </c>
-      <c r="I291" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="J291" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="K291" t="n">
-        <v>6.91</v>
-      </c>
-      <c r="L291" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="M291" t="n">
-        <v>7.29</v>
-      </c>
-      <c r="N291" t="n">
-        <v>6.04</v>
-      </c>
-      <c r="O291" t="n">
-        <v>5.403</v>
-      </c>
-      <c r="P291" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q291" t="n">
-        <v>0.3575</v>
-      </c>
-      <c r="R291" t="n">
-        <v>2.707</v>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="n">
-        <v>96</v>
-      </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
-        </is>
-      </c>
-      <c r="C292" t="inlineStr">
-        <is>
-          <t>McKeesport, PA</t>
-        </is>
-      </c>
-      <c r="D292" t="n">
-        <v>220</v>
-      </c>
-      <c r="E292" t="inlineStr">
-        <is>
-          <t>dryer</t>
-        </is>
-      </c>
-      <c r="F292" t="n">
-        <v>7</v>
-      </c>
-      <c r="G292" t="inlineStr">
-        <is>
-          <t>Townhouse</t>
-        </is>
-      </c>
-      <c r="H292" t="n">
-        <v>4</v>
-      </c>
-      <c r="I292" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="J292" t="inlineStr">
-        <is>
-          <t>10:00 PM</t>
-        </is>
-      </c>
-      <c r="K292" t="n">
-        <v>6.91</v>
-      </c>
-      <c r="L292" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="M292" t="n">
-        <v>3.36</v>
-      </c>
-      <c r="N292" t="n">
-        <v>3.11</v>
-      </c>
-      <c r="O292" t="n">
-        <v>4.1775</v>
-      </c>
-      <c r="P292" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q292" t="n">
-        <v>0.3575</v>
-      </c>
-      <c r="R292" t="n">
-        <v>2.707</v>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="n">
-        <v>97</v>
-      </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
-        </is>
-      </c>
-      <c r="C293" t="inlineStr">
-        <is>
-          <t>Harrisburg, PA</t>
-        </is>
-      </c>
-      <c r="D293" t="n">
-        <v>200</v>
-      </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>dishwasher</t>
-        </is>
-      </c>
-      <c r="F293" t="n">
-        <v>10</v>
-      </c>
-      <c r="G293" t="inlineStr">
-        <is>
-          <t>Single-family</t>
-        </is>
-      </c>
-      <c r="H293" t="n">
-        <v>6</v>
-      </c>
-      <c r="I293" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="J293" t="inlineStr">
-        <is>
-          <t>6:00 PM</t>
-        </is>
-      </c>
-      <c r="K293" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="L293" t="n">
-        <v>5.51</v>
-      </c>
-      <c r="M293" t="n">
-        <v>10</v>
-      </c>
-      <c r="N293" t="n">
-        <v>10</v>
-      </c>
-      <c r="O293" t="n">
-        <v>8.0115</v>
-      </c>
-      <c r="P293" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q293" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="R293" t="n">
-        <v>1.77</v>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="n">
-        <v>97</v>
-      </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
-        </is>
-      </c>
-      <c r="C294" t="inlineStr">
-        <is>
-          <t>Harrisburg, PA</t>
-        </is>
-      </c>
-      <c r="D294" t="n">
-        <v>200</v>
-      </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>dishwasher</t>
-        </is>
-      </c>
-      <c r="F294" t="n">
-        <v>10</v>
-      </c>
-      <c r="G294" t="inlineStr">
-        <is>
-          <t>Single-family</t>
-        </is>
-      </c>
-      <c r="H294" t="n">
-        <v>6</v>
-      </c>
-      <c r="I294" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="J294" t="inlineStr">
-        <is>
-          <t>9:00 AM</t>
-        </is>
-      </c>
-      <c r="K294" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="L294" t="n">
-        <v>5.51</v>
-      </c>
-      <c r="M294" t="n">
-        <v>5.21</v>
-      </c>
-      <c r="N294" t="n">
-        <v>4.64</v>
-      </c>
-      <c r="O294" t="n">
-        <v>6.249499999999999</v>
-      </c>
-      <c r="P294" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q294" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="R294" t="n">
-        <v>1.77</v>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="n">
-        <v>97</v>
-      </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
-        </is>
-      </c>
-      <c r="C295" t="inlineStr">
-        <is>
-          <t>Harrisburg, PA</t>
-        </is>
-      </c>
-      <c r="D295" t="n">
-        <v>200</v>
-      </c>
-      <c r="E295" t="inlineStr">
-        <is>
-          <t>dishwasher</t>
-        </is>
-      </c>
-      <c r="F295" t="n">
-        <v>10</v>
-      </c>
-      <c r="G295" t="inlineStr">
-        <is>
-          <t>Single-family</t>
-        </is>
-      </c>
-      <c r="H295" t="n">
-        <v>6</v>
-      </c>
-      <c r="I295" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="J295" t="inlineStr">
-        <is>
-          <t>10:00 PM</t>
-        </is>
-      </c>
-      <c r="K295" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="L295" t="n">
-        <v>5.51</v>
-      </c>
-      <c r="M295" t="n">
-        <v>7.83</v>
-      </c>
-      <c r="N295" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="O295" t="n">
-        <v>6.933999999999999</v>
-      </c>
-      <c r="P295" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q295" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="R295" t="n">
         <v>1.77</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added scenarios to get rounded counts
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_appliance.xlsx
+++ b/Ground Truth/ground_truth_appliance.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R289"/>
+  <dimension ref="A1:R301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,7 +444,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>appliance_age_type</t>
+          <t>appliance_age</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -18726,50 +18726,50 @@
     </row>
     <row r="278">
       <c r="A278" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
+          <t>It's around 8 in the morning and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Pottstown, PA</t>
+          <t>Levittown, PA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>washing_machine</t>
+          <t>dishwasher</t>
         </is>
       </c>
       <c r="F278" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="H278" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I278" t="n">
-        <v>0.3</v>
+        <v>0.85</v>
       </c>
       <c r="J278" t="inlineStr">
         <is>
-          <t>3:00 PM</t>
+          <t>8:00 AM</t>
         </is>
       </c>
       <c r="K278" t="n">
-        <v>9.279999999999999</v>
+        <v>10</v>
       </c>
       <c r="L278" t="n">
-        <v>9.800000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M278" t="n">
         <v>10</v>
@@ -18778,64 +18778,64 @@
         <v>10</v>
       </c>
       <c r="O278" t="n">
-        <v>9.714</v>
+        <v>9.341999999999999</v>
       </c>
       <c r="P278" t="n">
         <v>1</v>
       </c>
       <c r="Q278" t="n">
-        <v>0.096</v>
+        <v>0</v>
       </c>
       <c r="R278" t="n">
-        <v>0.312</v>
+        <v>0.885</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
+          <t>It's around 8 in the morning and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Pottstown, PA</t>
+          <t>Levittown, PA</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>washing_machine</t>
+          <t>dishwasher</t>
         </is>
       </c>
       <c r="F279" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="H279" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I279" t="n">
-        <v>0.3</v>
+        <v>0.85</v>
       </c>
       <c r="J279" t="inlineStr">
         <is>
-          <t>9:00 PM</t>
+          <t>2:00 PM</t>
         </is>
       </c>
       <c r="K279" t="n">
-        <v>9.949999999999999</v>
+        <v>10</v>
       </c>
       <c r="L279" t="n">
-        <v>9.800000000000001</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="M279" t="n">
         <v>7.43</v>
@@ -18844,130 +18844,130 @@
         <v>6.21</v>
       </c>
       <c r="O279" t="n">
-        <v>8.8325</v>
+        <v>8.259499999999999</v>
       </c>
       <c r="P279" t="n">
         <v>2</v>
       </c>
       <c r="Q279" t="n">
-        <v>0.0228</v>
+        <v>0</v>
       </c>
       <c r="R279" t="n">
-        <v>0.312</v>
+        <v>0.885</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
+          <t>It's around 8 in the morning and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Pottstown, PA</t>
+          <t>Levittown, PA</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>washing_machine</t>
+          <t>dishwasher</t>
         </is>
       </c>
       <c r="F280" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="H280" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I280" t="n">
-        <v>0.3</v>
+        <v>0.85</v>
       </c>
       <c r="J280" t="inlineStr">
         <is>
-          <t>6:00 AM</t>
+          <t>11:00 PM</t>
         </is>
       </c>
       <c r="K280" t="n">
-        <v>9.949999999999999</v>
+        <v>10</v>
       </c>
       <c r="L280" t="n">
-        <v>9.859999999999999</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="M280" t="n">
-        <v>4.71</v>
+        <v>6.29</v>
       </c>
       <c r="N280" t="n">
-        <v>4.78</v>
+        <v>3.63</v>
       </c>
       <c r="O280" t="n">
-        <v>8.095000000000001</v>
+        <v>7.7005</v>
       </c>
       <c r="P280" t="n">
         <v>3</v>
       </c>
       <c r="Q280" t="n">
-        <v>0.0228</v>
+        <v>0</v>
       </c>
       <c r="R280" t="n">
-        <v>0.293</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Phoenixville, PA</t>
+          <t>Pottstown, PA</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>dryer</t>
+          <t>washing_machine</t>
         </is>
       </c>
       <c r="F281" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Townhouse</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H281" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I281" t="n">
-        <v>2.8</v>
+        <v>0.3</v>
       </c>
       <c r="J281" t="inlineStr">
         <is>
-          <t>7:00 PM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="K281" t="n">
-        <v>8.220000000000001</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="L281" t="n">
-        <v>2.14</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M281" t="n">
         <v>10</v>
@@ -18976,166 +18976,166 @@
         <v>10</v>
       </c>
       <c r="O281" t="n">
-        <v>6.715</v>
+        <v>9.714</v>
       </c>
       <c r="P281" t="n">
         <v>1</v>
       </c>
       <c r="Q281" t="n">
-        <v>0.2128</v>
+        <v>0.096</v>
       </c>
       <c r="R281" t="n">
-        <v>2.915</v>
+        <v>0.312</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Phoenixville, PA</t>
+          <t>Pottstown, PA</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>dryer</t>
+          <t>washing_machine</t>
         </is>
       </c>
       <c r="F282" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Townhouse</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H282" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I282" t="n">
-        <v>2.8</v>
+        <v>0.3</v>
       </c>
       <c r="J282" t="inlineStr">
         <is>
-          <t>11:00 PM</t>
+          <t>9:00 PM</t>
         </is>
       </c>
       <c r="K282" t="n">
-        <v>8.220000000000001</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="L282" t="n">
-        <v>2.68</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="M282" t="n">
-        <v>6.2</v>
+        <v>7.43</v>
       </c>
       <c r="N282" t="n">
         <v>6.21</v>
       </c>
       <c r="O282" t="n">
-        <v>5.5755</v>
+        <v>8.8325</v>
       </c>
       <c r="P282" t="n">
         <v>2</v>
       </c>
       <c r="Q282" t="n">
-        <v>0.2128</v>
+        <v>0.0228</v>
       </c>
       <c r="R282" t="n">
-        <v>2.733</v>
+        <v>0.312</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's about 3 in the afternoon and I need to run the washing machine. When should I start it?</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Phoenixville, PA</t>
+          <t>Pottstown, PA</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>dryer</t>
+          <t>washing_machine</t>
         </is>
       </c>
       <c r="F283" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Townhouse</t>
+          <t>Single-family</t>
         </is>
       </c>
       <c r="H283" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I283" t="n">
-        <v>2.8</v>
+        <v>0.3</v>
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>8:00 AM</t>
+          <t>6:00 AM</t>
         </is>
       </c>
       <c r="K283" t="n">
-        <v>8.220000000000001</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="L283" t="n">
-        <v>2.14</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="M283" t="n">
-        <v>5.53</v>
+        <v>4.71</v>
       </c>
       <c r="N283" t="n">
-        <v>3.93</v>
+        <v>4.78</v>
       </c>
       <c r="O283" t="n">
-        <v>4.910500000000001</v>
+        <v>8.095000000000001</v>
       </c>
       <c r="P283" t="n">
         <v>3</v>
       </c>
       <c r="Q283" t="n">
-        <v>0.2128</v>
+        <v>0.0228</v>
       </c>
       <c r="R283" t="n">
-        <v>2.915</v>
+        <v>0.293</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>McKeesport, PA</t>
+          <t>Phoenixville, PA</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>220</v>
+        <v>155</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -19143,7 +19143,7 @@
         </is>
       </c>
       <c r="F284" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G284" t="inlineStr">
         <is>
@@ -19151,21 +19151,21 @@
         </is>
       </c>
       <c r="H284" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I284" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="J284" t="inlineStr">
         <is>
-          <t>2:00 PM</t>
+          <t>7:00 PM</t>
         </is>
       </c>
       <c r="K284" t="n">
-        <v>6.91</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="L284" t="n">
-        <v>2.76</v>
+        <v>2.14</v>
       </c>
       <c r="M284" t="n">
         <v>10</v>
@@ -19174,34 +19174,34 @@
         <v>10</v>
       </c>
       <c r="O284" t="n">
-        <v>6.539</v>
+        <v>6.715</v>
       </c>
       <c r="P284" t="n">
         <v>1</v>
       </c>
       <c r="Q284" t="n">
-        <v>0.3575</v>
+        <v>0.2128</v>
       </c>
       <c r="R284" t="n">
-        <v>2.707</v>
+        <v>2.915</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>McKeesport, PA</t>
+          <t>Phoenixville, PA</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>220</v>
+        <v>155</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -19209,7 +19209,7 @@
         </is>
       </c>
       <c r="F285" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G285" t="inlineStr">
         <is>
@@ -19217,57 +19217,57 @@
         </is>
       </c>
       <c r="H285" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I285" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="J285" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>11:00 PM</t>
         </is>
       </c>
       <c r="K285" t="n">
-        <v>6.91</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="L285" t="n">
-        <v>2.76</v>
+        <v>2.68</v>
       </c>
       <c r="M285" t="n">
-        <v>7.29</v>
+        <v>6.2</v>
       </c>
       <c r="N285" t="n">
-        <v>6.04</v>
+        <v>6.21</v>
       </c>
       <c r="O285" t="n">
-        <v>5.403</v>
+        <v>5.5755</v>
       </c>
       <c r="P285" t="n">
         <v>2</v>
       </c>
       <c r="Q285" t="n">
-        <v>0.3575</v>
+        <v>0.2128</v>
       </c>
       <c r="R285" t="n">
-        <v>2.707</v>
+        <v>2.733</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's just past 7 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>McKeesport, PA</t>
+          <t>Phoenixville, PA</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>220</v>
+        <v>155</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -19275,7 +19275,7 @@
         </is>
       </c>
       <c r="F286" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G286" t="inlineStr">
         <is>
@@ -19283,57 +19283,57 @@
         </is>
       </c>
       <c r="H286" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I286" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="J286" t="inlineStr">
         <is>
-          <t>10:00 PM</t>
+          <t>8:00 AM</t>
         </is>
       </c>
       <c r="K286" t="n">
-        <v>6.91</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="L286" t="n">
-        <v>2.76</v>
+        <v>2.14</v>
       </c>
       <c r="M286" t="n">
-        <v>3.36</v>
+        <v>5.53</v>
       </c>
       <c r="N286" t="n">
-        <v>3.11</v>
+        <v>3.93</v>
       </c>
       <c r="O286" t="n">
-        <v>4.1775</v>
+        <v>4.910500000000001</v>
       </c>
       <c r="P286" t="n">
         <v>3</v>
       </c>
       <c r="Q286" t="n">
-        <v>0.3575</v>
+        <v>0.2128</v>
       </c>
       <c r="R286" t="n">
-        <v>2.707</v>
+        <v>2.915</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>It's around 11 in the morning and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Harrisburg, PA</t>
+          <t>Quakertown, PA</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -19341,29 +19341,29 @@
         </is>
       </c>
       <c r="F287" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="H287" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I287" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>6:00 PM</t>
+          <t>11:00 AM</t>
         </is>
       </c>
       <c r="K287" t="n">
-        <v>8.609999999999999</v>
+        <v>10</v>
       </c>
       <c r="L287" t="n">
-        <v>5.51</v>
+        <v>7.35</v>
       </c>
       <c r="M287" t="n">
         <v>10</v>
@@ -19372,34 +19372,34 @@
         <v>10</v>
       </c>
       <c r="O287" t="n">
-        <v>8.0115</v>
+        <v>9.0725</v>
       </c>
       <c r="P287" t="n">
         <v>1</v>
       </c>
       <c r="Q287" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="R287" t="n">
-        <v>1.77</v>
+        <v>1.145</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>It's around 11 in the morning and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Harrisburg, PA</t>
+          <t>Quakertown, PA</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -19407,113 +19407,905 @@
         </is>
       </c>
       <c r="F288" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Single-family</t>
+          <t>Apartment</t>
         </is>
       </c>
       <c r="H288" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I288" t="n">
-        <v>1.7</v>
+        <v>1.1</v>
       </c>
       <c r="J288" t="inlineStr">
         <is>
-          <t>9:00 AM</t>
+          <t>3:00 PM</t>
         </is>
       </c>
       <c r="K288" t="n">
-        <v>8.609999999999999</v>
+        <v>10</v>
       </c>
       <c r="L288" t="n">
-        <v>5.51</v>
+        <v>7.35</v>
       </c>
       <c r="M288" t="n">
-        <v>5.21</v>
+        <v>8.23</v>
       </c>
       <c r="N288" t="n">
-        <v>4.64</v>
+        <v>7.15</v>
       </c>
       <c r="O288" t="n">
-        <v>6.249499999999999</v>
+        <v>8.291</v>
       </c>
       <c r="P288" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q288" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="R288" t="n">
-        <v>1.77</v>
+        <v>1.145</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
+        <v>95</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>It's around 11 in the morning and I need to run the dishwasher. When should I start it?</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Quakertown, PA</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>140</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>dishwasher</t>
+        </is>
+      </c>
+      <c r="F289" t="n">
+        <v>4</v>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>Apartment</t>
+        </is>
+      </c>
+      <c r="H289" t="n">
+        <v>2</v>
+      </c>
+      <c r="I289" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>10:00 PM</t>
+        </is>
+      </c>
+      <c r="K289" t="n">
+        <v>10</v>
+      </c>
+      <c r="L289" t="n">
+        <v>7.35</v>
+      </c>
+      <c r="M289" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="N289" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="O289" t="n">
+        <v>7.0835</v>
+      </c>
+      <c r="P289" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q289" t="n">
+        <v>0</v>
+      </c>
+      <c r="R289" t="n">
+        <v>1.145</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>96</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>McKeesport, PA</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>220</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>dryer</t>
+        </is>
+      </c>
+      <c r="F290" t="n">
+        <v>7</v>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>Townhouse</t>
+        </is>
+      </c>
+      <c r="H290" t="n">
+        <v>4</v>
+      </c>
+      <c r="I290" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>2:00 PM</t>
+        </is>
+      </c>
+      <c r="K290" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="L290" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="M290" t="n">
+        <v>10</v>
+      </c>
+      <c r="N290" t="n">
+        <v>10</v>
+      </c>
+      <c r="O290" t="n">
+        <v>6.539</v>
+      </c>
+      <c r="P290" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q290" t="n">
+        <v>0.3575</v>
+      </c>
+      <c r="R290" t="n">
+        <v>2.707</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>96</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>McKeesport, PA</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>220</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>dryer</t>
+        </is>
+      </c>
+      <c r="F291" t="n">
+        <v>7</v>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>Townhouse</t>
+        </is>
+      </c>
+      <c r="H291" t="n">
+        <v>4</v>
+      </c>
+      <c r="I291" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="K291" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="L291" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="M291" t="n">
+        <v>7.29</v>
+      </c>
+      <c r="N291" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="O291" t="n">
+        <v>5.403</v>
+      </c>
+      <c r="P291" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q291" t="n">
+        <v>0.3575</v>
+      </c>
+      <c r="R291" t="n">
+        <v>2.707</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>96</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>McKeesport, PA</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>220</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>dryer</t>
+        </is>
+      </c>
+      <c r="F292" t="n">
+        <v>7</v>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>Townhouse</t>
+        </is>
+      </c>
+      <c r="H292" t="n">
+        <v>4</v>
+      </c>
+      <c r="I292" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>10:00 PM</t>
+        </is>
+      </c>
+      <c r="K292" t="n">
+        <v>6.91</v>
+      </c>
+      <c r="L292" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="M292" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="N292" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="O292" t="n">
+        <v>4.1775</v>
+      </c>
+      <c r="P292" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q292" t="n">
+        <v>0.3575</v>
+      </c>
+      <c r="R292" t="n">
+        <v>2.707</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
         <v>97</v>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B293" t="inlineStr">
         <is>
           <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
-      <c r="C289" t="inlineStr">
+      <c r="C293" t="inlineStr">
         <is>
           <t>Harrisburg, PA</t>
         </is>
       </c>
-      <c r="D289" t="n">
+      <c r="D293" t="n">
         <v>200</v>
       </c>
-      <c r="E289" t="inlineStr">
+      <c r="E293" t="inlineStr">
         <is>
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F289" t="n">
-        <v>10</v>
-      </c>
-      <c r="G289" t="inlineStr">
+      <c r="F293" t="n">
+        <v>10</v>
+      </c>
+      <c r="G293" t="inlineStr">
         <is>
           <t>Single-family</t>
         </is>
       </c>
-      <c r="H289" t="n">
+      <c r="H293" t="n">
         <v>6</v>
       </c>
-      <c r="I289" t="n">
+      <c r="I293" t="n">
         <v>1.7</v>
       </c>
-      <c r="J289" t="inlineStr">
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>6:00 PM</t>
+        </is>
+      </c>
+      <c r="K293" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="L293" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="M293" t="n">
+        <v>10</v>
+      </c>
+      <c r="N293" t="n">
+        <v>10</v>
+      </c>
+      <c r="O293" t="n">
+        <v>8.0115</v>
+      </c>
+      <c r="P293" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q293" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="R293" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>97</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Harrisburg, PA</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>200</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>dishwasher</t>
+        </is>
+      </c>
+      <c r="F294" t="n">
+        <v>10</v>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>Single-family</t>
+        </is>
+      </c>
+      <c r="H294" t="n">
+        <v>6</v>
+      </c>
+      <c r="I294" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>9:00 AM</t>
+        </is>
+      </c>
+      <c r="K294" t="n">
+        <v>8.609999999999999</v>
+      </c>
+      <c r="L294" t="n">
+        <v>5.51</v>
+      </c>
+      <c r="M294" t="n">
+        <v>5.21</v>
+      </c>
+      <c r="N294" t="n">
+        <v>4.64</v>
+      </c>
+      <c r="O294" t="n">
+        <v>6.249499999999999</v>
+      </c>
+      <c r="P294" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q294" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="R294" t="n">
+        <v>1.77</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>97</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Harrisburg, PA</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>200</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>dishwasher</t>
+        </is>
+      </c>
+      <c r="F295" t="n">
+        <v>10</v>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>Single-family</t>
+        </is>
+      </c>
+      <c r="H295" t="n">
+        <v>6</v>
+      </c>
+      <c r="I295" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J295" t="inlineStr">
         <is>
           <t>10:00 PM</t>
         </is>
       </c>
-      <c r="K289" t="n">
+      <c r="K295" t="n">
         <v>8.609999999999999</v>
       </c>
-      <c r="L289" t="n">
+      <c r="L295" t="n">
         <v>5.51</v>
       </c>
-      <c r="M289" t="n">
+      <c r="M295" t="n">
         <v>7.83</v>
       </c>
-      <c r="N289" t="n">
+      <c r="N295" t="n">
         <v>5.71</v>
       </c>
-      <c r="O289" t="n">
+      <c r="O295" t="n">
         <v>6.933999999999999</v>
       </c>
-      <c r="P289" t="n">
+      <c r="P295" t="n">
         <v>2</v>
       </c>
-      <c r="Q289" t="n">
+      <c r="Q295" t="n">
         <v>0.17</v>
       </c>
-      <c r="R289" t="n">
+      <c r="R295" t="n">
         <v>1.77</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>98</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Laundry finished around 6 PM in Harrisburg. When should I run the dryer?</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Harrisburg, PA</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>260</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Dryer</t>
+        </is>
+      </c>
+      <c r="F296" t="n">
+        <v>9</v>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>Rowhouse</t>
+        </is>
+      </c>
+      <c r="H296" t="n">
+        <v>4</v>
+      </c>
+      <c r="I296" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>6pm</t>
+        </is>
+      </c>
+      <c r="K296" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="L296" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="M296" t="n">
+        <v>10</v>
+      </c>
+      <c r="N296" t="n">
+        <v>10</v>
+      </c>
+      <c r="O296" t="n">
+        <v>7.0735</v>
+      </c>
+      <c r="P296" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q296" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="R296" t="n">
+        <v>2.498</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>98</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Laundry finished around 6 PM in Harrisburg. When should I run the dryer?</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Harrisburg, PA</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>260</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Dryer</t>
+        </is>
+      </c>
+      <c r="F297" t="n">
+        <v>9</v>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>Rowhouse</t>
+        </is>
+      </c>
+      <c r="H297" t="n">
+        <v>4</v>
+      </c>
+      <c r="I297" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>10pm</t>
+        </is>
+      </c>
+      <c r="K297" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="L297" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="M297" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="N297" t="n">
+        <v>5.67</v>
+      </c>
+      <c r="O297" t="n">
+        <v>5.562</v>
+      </c>
+      <c r="P297" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q297" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="R297" t="n">
+        <v>2.498</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>98</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Laundry finished around 6 PM in Harrisburg. When should I run the dryer?</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Harrisburg, PA</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>260</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Dryer</t>
+        </is>
+      </c>
+      <c r="F298" t="n">
+        <v>9</v>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>Rowhouse</t>
+        </is>
+      </c>
+      <c r="H298" t="n">
+        <v>4</v>
+      </c>
+      <c r="I298" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>6am</t>
+        </is>
+      </c>
+      <c r="K298" t="n">
+        <v>7.98</v>
+      </c>
+      <c r="L298" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="M298" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="N298" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="O298" t="n">
+        <v>4.353</v>
+      </c>
+      <c r="P298" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q298" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="R298" t="n">
+        <v>2.342</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>99</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>It's around 8 in the morning and I need to run the dishwasher in Doylestown. When should I start it?</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Doylestown, PA</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>210</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Dishwasher</t>
+        </is>
+      </c>
+      <c r="F299" t="n">
+        <v>6</v>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>Townhouse</t>
+        </is>
+      </c>
+      <c r="H299" t="n">
+        <v>3</v>
+      </c>
+      <c r="I299" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>8am</t>
+        </is>
+      </c>
+      <c r="K299" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="L299" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M299" t="n">
+        <v>10</v>
+      </c>
+      <c r="N299" t="n">
+        <v>10</v>
+      </c>
+      <c r="O299" t="n">
+        <v>8.954000000000001</v>
+      </c>
+      <c r="P299" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q299" t="n">
+        <v>0.0798</v>
+      </c>
+      <c r="R299" t="n">
+        <v>1.093</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>99</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>It's around 8 in the morning and I need to run the dishwasher in Doylestown. When should I start it?</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Doylestown, PA</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>210</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Dishwasher</t>
+        </is>
+      </c>
+      <c r="F300" t="n">
+        <v>6</v>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>Townhouse</t>
+        </is>
+      </c>
+      <c r="H300" t="n">
+        <v>3</v>
+      </c>
+      <c r="I300" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>2pm</t>
+        </is>
+      </c>
+      <c r="K300" t="n">
+        <v>7.11</v>
+      </c>
+      <c r="L300" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="M300" t="n">
+        <v>7.09</v>
+      </c>
+      <c r="N300" t="n">
+        <v>5.81</v>
+      </c>
+      <c r="O300" t="n">
+        <v>7.0475</v>
+      </c>
+      <c r="P300" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q300" t="n">
+        <v>0.336</v>
+      </c>
+      <c r="R300" t="n">
+        <v>1.093</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>99</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>It's around 8 in the morning and I need to run the dishwasher in Doylestown. When should I start it?</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Doylestown, PA</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>210</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Dishwasher</t>
+        </is>
+      </c>
+      <c r="F301" t="n">
+        <v>6</v>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>Townhouse</t>
+        </is>
+      </c>
+      <c r="H301" t="n">
+        <v>3</v>
+      </c>
+      <c r="I301" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>11pm</t>
+        </is>
+      </c>
+      <c r="K301" t="n">
+        <v>9.43</v>
+      </c>
+      <c r="L301" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="M301" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="N301" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="O301" t="n">
+        <v>7.103499999999999</v>
+      </c>
+      <c r="P301" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q301" t="n">
+        <v>0.0798</v>
+      </c>
+      <c r="R301" t="n">
+        <v>1.025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
c hanged reading and writing and some formatting issues
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_appliance.xlsx
+++ b/Ground Truth/ground_truth_appliance.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Regenerate ground truth from normalized scenario inputs
Re-ran all 3 GT calculators against the canonical-header scenario files.
- Outputs now carry canonical headers (question, household_size, ...).
- Appliance GT picks up the corruption + grammar + appliance-name fixes.
- MAVT ordering verified correct: rank 1 = max weighted MAVT, ranks are
  clean 1..3 permutations, order matches deterministic tie-breaks,
  recomputed MAVT matches stored (0 mismatches across all 3 files).
- Row counts unchanged: HVAC 315, Appliance 300, Shower 240.

Known pre-existing data gap (NOT introduced here, identical at HEAD):
appliance scenarios 92 (Levittown) and 95 (Quakertown) have cities absent
from CITY_TO_UTILITY, so their energy_cost falls back to 0. Flagged for a
follow-up decision on the correct utility mapping.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_appliance.xlsx
+++ b/Ground Truth/ground_truth_appliance.xlsx
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>question</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>occupants</t>
+          <t>household_size</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -530,8 +530,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>8</v>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -596,8 +598,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>8</v>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -662,8 +666,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F4" t="n">
-        <v>8</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -728,8 +734,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F5" t="n">
-        <v>12</v>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -794,8 +802,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F6" t="n">
-        <v>12</v>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -860,8 +870,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F7" t="n">
-        <v>12</v>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -926,8 +938,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F8" t="n">
-        <v>6</v>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -992,8 +1006,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F9" t="n">
-        <v>6</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1058,8 +1074,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F10" t="n">
-        <v>6</v>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1121,11 +1139,13 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F11" t="n">
-        <v>3</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1187,11 +1207,13 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F12" t="n">
-        <v>3</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1253,11 +1275,13 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>3</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1306,7 +1330,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>It's just past 5 PM � when should I run the dryer?</t>
+          <t>It's just past 5 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1322,8 +1346,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F14" t="n">
-        <v>15</v>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1372,7 +1398,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>It's just past 5 PM � when should I run the dryer?</t>
+          <t>It's just past 5 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1388,8 +1414,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F15" t="n">
-        <v>15</v>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1438,7 +1466,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>It's just past 5 PM � when should I run the dryer?</t>
+          <t>It's just past 5 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1454,8 +1482,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F16" t="n">
-        <v>15</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1520,8 +1550,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F17" t="n">
-        <v>10</v>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1586,8 +1618,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F18" t="n">
-        <v>10</v>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1652,8 +1686,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F19" t="n">
-        <v>10</v>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1718,8 +1754,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F20" t="n">
-        <v>7</v>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1784,8 +1822,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F21" t="n">
-        <v>7</v>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1850,8 +1890,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F22" t="n">
-        <v>7</v>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1916,8 +1958,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F23" t="n">
-        <v>7</v>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1982,8 +2026,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F24" t="n">
-        <v>7</v>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -2048,8 +2094,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F25" t="n">
-        <v>7</v>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -2114,8 +2162,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F26" t="n">
-        <v>10</v>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -2180,8 +2230,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F27" t="n">
-        <v>10</v>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -2246,8 +2298,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F28" t="n">
-        <v>10</v>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -2296,7 +2350,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>It's around 7 in the evening � when should I run the dishwasher?</t>
+          <t>It's around 7 in the evening — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2312,8 +2366,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>2</v>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -2362,7 +2418,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>It's around 7 in the evening � when should I run the dishwasher?</t>
+          <t>It's around 7 in the evening — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2378,8 +2434,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F30" t="n">
-        <v>2</v>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -2428,7 +2486,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>It's around 7 in the evening � when should I run the dishwasher?</t>
+          <t>It's around 7 in the evening — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2444,8 +2502,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F31" t="n">
-        <v>2</v>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -2510,8 +2570,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F32" t="n">
-        <v>6</v>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2576,8 +2638,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>6</v>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -2642,8 +2706,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F34" t="n">
-        <v>6</v>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -2708,8 +2774,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>4</v>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -2774,8 +2842,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F36" t="n">
-        <v>4</v>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -2840,8 +2910,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>4</v>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -2906,8 +2978,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F38" t="n">
-        <v>6</v>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2972,8 +3046,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>6</v>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -3038,8 +3114,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F40" t="n">
-        <v>6</v>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -3104,8 +3182,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>12</v>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -3170,8 +3250,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F42" t="n">
-        <v>12</v>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -3236,8 +3318,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F43" t="n">
-        <v>12</v>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -3302,8 +3386,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F44" t="n">
-        <v>8</v>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -3368,8 +3454,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F45" t="n">
-        <v>8</v>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -3434,8 +3522,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F46" t="n">
-        <v>8</v>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -3484,7 +3574,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3500,8 +3590,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F47" t="n">
-        <v>6</v>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -3550,7 +3642,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3566,8 +3658,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F48" t="n">
-        <v>6</v>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -3616,7 +3710,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3632,8 +3726,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>6</v>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -3682,7 +3778,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>It's just past 5 PM � when should I run the washer?</t>
+          <t>It's just past 5 PM — when should I run the washer?</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3695,11 +3791,13 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F50" t="n">
-        <v>10</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -3748,7 +3846,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>It's just past 5 PM � when should I run the washer?</t>
+          <t>It's just past 5 PM — when should I run the washer?</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3761,11 +3859,13 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>10</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -3814,7 +3914,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>It's just past 5 PM � when should I run the washer?</t>
+          <t>It's just past 5 PM — when should I run the washer?</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3827,11 +3927,13 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F52" t="n">
-        <v>10</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -3896,8 +3998,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F53" t="n">
-        <v>12</v>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -3962,8 +4066,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F54" t="n">
-        <v>12</v>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -4028,8 +4134,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F55" t="n">
-        <v>12</v>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -4094,8 +4202,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F56" t="n">
-        <v>7</v>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -4160,8 +4270,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>7</v>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4226,8 +4338,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F58" t="n">
-        <v>7</v>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4292,8 +4406,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F59" t="n">
-        <v>15</v>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -4358,8 +4474,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F60" t="n">
-        <v>15</v>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -4424,8 +4542,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F61" t="n">
-        <v>15</v>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -4490,8 +4610,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F62" t="n">
-        <v>2</v>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -4556,8 +4678,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F63" t="n">
-        <v>2</v>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -4622,8 +4746,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F64" t="n">
-        <v>2</v>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -4688,8 +4814,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F65" t="n">
-        <v>4</v>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -4754,8 +4882,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F66" t="n">
-        <v>4</v>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -4820,8 +4950,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F67" t="n">
-        <v>4</v>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -4886,8 +5018,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F68" t="n">
-        <v>15</v>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -4952,8 +5086,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F69" t="n">
-        <v>15</v>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -5018,8 +5154,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F70" t="n">
-        <v>15</v>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -5084,8 +5222,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F71" t="n">
-        <v>6</v>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -5150,8 +5290,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F72" t="n">
-        <v>6</v>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -5216,8 +5358,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F73" t="n">
-        <v>6</v>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -5266,7 +5410,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>It's past 1 in the morning � when should I run the dryer?</t>
+          <t>It's past 1 in the morning — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5282,8 +5426,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F74" t="n">
-        <v>12</v>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -5332,7 +5478,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>It's past 1 in the morning � when should I run the dryer?</t>
+          <t>It's past 1 in the morning — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -5348,8 +5494,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>12</v>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -5398,7 +5546,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>It's past 1 in the morning � when should I run the dryer?</t>
+          <t>It's past 1 in the morning — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -5414,8 +5562,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F76" t="n">
-        <v>12</v>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -5477,11 +5627,13 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F77" t="n">
-        <v>8</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -5543,11 +5695,13 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F78" t="n">
-        <v>8</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -5609,11 +5763,13 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F79" t="n">
-        <v>8</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -5678,8 +5834,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F80" t="n">
-        <v>10</v>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -5744,8 +5902,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>10</v>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -5810,8 +5970,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F82" t="n">
-        <v>10</v>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -5876,8 +6038,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F83" t="n">
-        <v>3</v>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -5942,8 +6106,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F84" t="n">
-        <v>3</v>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -6008,8 +6174,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F85" t="n">
-        <v>3</v>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -6058,7 +6226,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>It's just past midnight � when should I run the dishwasher?</t>
+          <t>It's just past midnight — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -6074,8 +6242,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F86" t="n">
-        <v>12</v>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -6124,7 +6294,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>It's just past midnight � when should I run the dishwasher?</t>
+          <t>It's just past midnight — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -6140,8 +6310,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F87" t="n">
-        <v>12</v>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -6190,7 +6362,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>It's just past midnight � when should I run the dishwasher?</t>
+          <t>It's just past midnight — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6206,8 +6378,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F88" t="n">
-        <v>12</v>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -6272,8 +6446,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F89" t="n">
-        <v>15</v>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -6338,8 +6514,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F90" t="n">
-        <v>15</v>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -6404,8 +6582,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F91" t="n">
-        <v>15</v>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -6470,8 +6650,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F92" t="n">
-        <v>2</v>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -6536,8 +6718,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F93" t="n">
-        <v>2</v>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -6602,8 +6786,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F94" t="n">
-        <v>2</v>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -6668,8 +6854,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F95" t="n">
-        <v>5</v>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -6734,8 +6922,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F96" t="n">
-        <v>5</v>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -6800,8 +6990,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F97" t="n">
-        <v>5</v>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -6866,8 +7058,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F98" t="n">
-        <v>6</v>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -6932,8 +7126,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F99" t="n">
-        <v>6</v>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -6998,8 +7194,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F100" t="n">
-        <v>6</v>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
@@ -7048,7 +7246,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>It's around 8 at night � when should I run the dishwasher?</t>
+          <t>It's around 8 at night — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -7064,8 +7262,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F101" t="n">
-        <v>4</v>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
@@ -7114,7 +7314,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>It's around 8 at night � when should I run the dishwasher?</t>
+          <t>It's around 8 at night — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -7130,8 +7330,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F102" t="n">
-        <v>4</v>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
@@ -7180,7 +7382,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>It's around 8 at night � when should I run the dishwasher?</t>
+          <t>It's around 8 at night — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -7196,8 +7398,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F103" t="n">
-        <v>4</v>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -7262,8 +7466,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F104" t="n">
-        <v>10</v>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -7328,8 +7534,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F105" t="n">
-        <v>10</v>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -7394,8 +7602,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F106" t="n">
-        <v>10</v>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -7457,11 +7667,13 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F107" t="n">
-        <v>2</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -7523,11 +7735,13 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F108" t="n">
-        <v>2</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -7589,11 +7803,13 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F109" t="n">
-        <v>2</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -7658,8 +7874,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F110" t="n">
-        <v>8</v>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -7724,8 +7942,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F111" t="n">
-        <v>8</v>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -7790,8 +8010,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F112" t="n">
-        <v>8</v>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -7853,11 +8075,13 @@
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F113" t="n">
-        <v>10</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -7919,11 +8143,13 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F114" t="n">
-        <v>10</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -7985,11 +8211,13 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F115" t="n">
-        <v>10</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -8051,11 +8279,13 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F116" t="n">
-        <v>6</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -8117,11 +8347,13 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F117" t="n">
-        <v>6</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -8183,11 +8415,13 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>washer</t>
-        </is>
-      </c>
-      <c r="F118" t="n">
-        <v>6</v>
+          <t>washing_machine</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -8252,8 +8486,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F119" t="n">
-        <v>6</v>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -8318,8 +8554,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F120" t="n">
-        <v>6</v>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -8384,8 +8622,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F121" t="n">
-        <v>6</v>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -8434,7 +8674,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -8450,8 +8690,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F122" t="n">
-        <v>8</v>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -8500,7 +8742,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -8516,8 +8758,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F123" t="n">
-        <v>8</v>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -8566,7 +8810,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -8582,8 +8826,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F124" t="n">
-        <v>8</v>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -8648,8 +8894,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F125" t="n">
-        <v>10</v>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -8714,8 +8962,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F126" t="n">
-        <v>10</v>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
@@ -8780,8 +9030,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F127" t="n">
-        <v>10</v>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -8846,8 +9098,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F128" t="n">
-        <v>5</v>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -8912,8 +9166,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F129" t="n">
-        <v>5</v>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
@@ -8978,8 +9234,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F130" t="n">
-        <v>5</v>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -9044,8 +9302,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F131" t="n">
-        <v>6</v>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -9110,8 +9370,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F132" t="n">
-        <v>6</v>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -9176,8 +9438,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F133" t="n">
-        <v>6</v>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -9242,8 +9506,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F134" t="n">
-        <v>4</v>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -9308,8 +9574,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F135" t="n">
-        <v>4</v>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -9374,8 +9642,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F136" t="n">
-        <v>4</v>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -9440,8 +9710,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F137" t="n">
-        <v>3</v>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -9506,8 +9778,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F138" t="n">
-        <v>3</v>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G138" t="inlineStr">
         <is>
@@ -9572,8 +9846,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F139" t="n">
-        <v>3</v>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -9638,8 +9914,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F140" t="n">
-        <v>7</v>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G140" t="inlineStr">
         <is>
@@ -9704,8 +9982,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F141" t="n">
-        <v>7</v>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G141" t="inlineStr">
         <is>
@@ -9770,8 +10050,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F142" t="n">
-        <v>7</v>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -9836,8 +10118,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F143" t="n">
-        <v>5</v>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -9902,8 +10186,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F144" t="n">
-        <v>5</v>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -9968,8 +10254,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F145" t="n">
-        <v>5</v>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -10034,8 +10322,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F146" t="n">
-        <v>4</v>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -10100,8 +10390,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F147" t="n">
-        <v>4</v>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -10166,8 +10458,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F148" t="n">
-        <v>4</v>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -10216,7 +10510,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -10232,8 +10526,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F149" t="n">
-        <v>6</v>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -10282,7 +10578,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -10298,8 +10594,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F150" t="n">
-        <v>6</v>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -10348,7 +10646,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>It's just past 9 AM � when should I run the dryer?</t>
+          <t>It's just past 9 AM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -10364,8 +10662,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F151" t="n">
-        <v>6</v>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -10430,8 +10730,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F152" t="n">
-        <v>8</v>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -10496,8 +10798,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F153" t="n">
-        <v>8</v>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -10562,8 +10866,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F154" t="n">
-        <v>8</v>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -10628,8 +10934,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F155" t="n">
-        <v>3</v>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -10694,8 +11002,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F156" t="n">
-        <v>3</v>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -10760,8 +11070,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F157" t="n">
-        <v>3</v>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -10826,8 +11138,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F158" t="n">
-        <v>2</v>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -10892,8 +11206,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F159" t="n">
-        <v>2</v>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -10958,8 +11274,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F160" t="n">
-        <v>2</v>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -11008,7 +11326,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening � when should I run the washing machine?</t>
+          <t>It's around 5 in the evening — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -11024,8 +11342,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F161" t="n">
-        <v>1</v>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -11074,7 +11394,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening � when should I run the washing machine?</t>
+          <t>It's around 5 in the evening — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -11090,8 +11410,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F162" t="n">
-        <v>1</v>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
@@ -11140,7 +11462,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening � when should I run the washing machine?</t>
+          <t>It's around 5 in the evening — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -11156,8 +11478,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F163" t="n">
-        <v>1</v>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -11222,8 +11546,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F164" t="n">
-        <v>15</v>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -11288,8 +11614,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F165" t="n">
-        <v>15</v>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -11354,8 +11682,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F166" t="n">
-        <v>15</v>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
@@ -11404,7 +11734,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>It's just past 7 PM � when should I run the dryer?</t>
+          <t>It's just past 7 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -11420,8 +11750,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F167" t="n">
-        <v>12</v>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -11470,7 +11802,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>It's just past 7 PM � when should I run the dryer?</t>
+          <t>It's just past 7 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -11486,8 +11818,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F168" t="n">
-        <v>12</v>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -11536,7 +11870,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>It's just past 7 PM � when should I run the dryer?</t>
+          <t>It's just past 7 PM — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -11552,8 +11886,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F169" t="n">
-        <v>12</v>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
       </c>
       <c r="G169" t="inlineStr">
         <is>
@@ -11618,8 +11954,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F170" t="n">
-        <v>2</v>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -11684,8 +12022,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F171" t="n">
-        <v>2</v>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -11750,8 +12090,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F172" t="n">
-        <v>2</v>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="G172" t="inlineStr">
         <is>
@@ -11816,8 +12158,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F173" t="n">
-        <v>5</v>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G173" t="inlineStr">
         <is>
@@ -11882,8 +12226,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F174" t="n">
-        <v>5</v>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -11948,8 +12294,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F175" t="n">
-        <v>5</v>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -11998,7 +12346,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>It's late � just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -12014,8 +12362,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F176" t="n">
-        <v>6</v>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G176" t="inlineStr">
         <is>
@@ -12064,7 +12414,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>It's late � just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -12080,8 +12430,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F177" t="n">
-        <v>6</v>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G177" t="inlineStr">
         <is>
@@ -12130,7 +12482,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>It's late � just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -12146,8 +12498,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F178" t="n">
-        <v>6</v>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -12212,8 +12566,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F179" t="n">
-        <v>4</v>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -12278,8 +12634,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F180" t="n">
-        <v>4</v>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -12344,8 +12702,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F181" t="n">
-        <v>4</v>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -12410,8 +12770,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F182" t="n">
-        <v>8</v>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -12476,8 +12838,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F183" t="n">
-        <v>8</v>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -12542,8 +12906,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F184" t="n">
-        <v>8</v>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -12592,7 +12958,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -12608,8 +12974,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F185" t="n">
-        <v>5</v>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -12658,7 +13026,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -12674,8 +13042,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F186" t="n">
-        <v>5</v>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -12724,7 +13094,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>It's getting close to midnight � when should I run the washing machine?</t>
+          <t>It's getting close to midnight — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -12740,8 +13110,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F187" t="n">
-        <v>5</v>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -12806,8 +13178,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F188" t="n">
-        <v>4</v>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -12872,8 +13246,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F189" t="n">
-        <v>4</v>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -12938,8 +13314,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F190" t="n">
-        <v>4</v>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -13004,8 +13382,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F191" t="n">
-        <v>7</v>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -13070,8 +13450,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F192" t="n">
-        <v>7</v>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -13136,8 +13518,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F193" t="n">
-        <v>7</v>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -13186,7 +13570,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>It's just after 8 AM � when should I run the dishwasher?</t>
+          <t>It's just after 8 AM — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -13202,8 +13586,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F194" t="n">
-        <v>5</v>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -13252,7 +13638,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>It's just after 8 AM � when should I run the dishwasher?</t>
+          <t>It's just after 8 AM — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -13268,8 +13654,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F195" t="n">
-        <v>5</v>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -13318,7 +13706,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>It's just after 8 AM � when should I run the dishwasher?</t>
+          <t>It's just after 8 AM — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -13334,8 +13722,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F196" t="n">
-        <v>5</v>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -13400,8 +13790,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F197" t="n">
-        <v>6</v>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -13466,8 +13858,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F198" t="n">
-        <v>6</v>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -13532,8 +13926,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F199" t="n">
-        <v>6</v>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -13598,8 +13994,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F200" t="n">
-        <v>5</v>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -13664,8 +14062,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F201" t="n">
-        <v>5</v>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -13730,8 +14130,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F202" t="n">
-        <v>5</v>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -13796,8 +14198,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F203" t="n">
-        <v>6</v>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -13862,8 +14266,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F204" t="n">
-        <v>6</v>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -13928,8 +14334,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F205" t="n">
-        <v>6</v>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -13994,8 +14402,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F206" t="n">
-        <v>4</v>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -14060,8 +14470,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F207" t="n">
-        <v>4</v>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -14126,8 +14538,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F208" t="n">
-        <v>4</v>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -14192,8 +14606,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F209" t="n">
-        <v>3</v>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -14258,8 +14674,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F210" t="n">
-        <v>3</v>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -14324,8 +14742,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F211" t="n">
-        <v>3</v>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -14390,8 +14810,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F212" t="n">
-        <v>1</v>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -14456,8 +14878,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F213" t="n">
-        <v>1</v>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -14522,8 +14946,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F214" t="n">
-        <v>1</v>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -14588,8 +15014,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F215" t="n">
-        <v>5</v>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -14654,8 +15082,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F216" t="n">
-        <v>5</v>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -14720,8 +15150,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F217" t="n">
-        <v>5</v>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -14770,7 +15202,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night � when should I run the washing machine?</t>
+          <t>It's nearly 11 at night — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -14786,8 +15218,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F218" t="n">
-        <v>6</v>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -14836,7 +15270,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night � when should I run the washing machine?</t>
+          <t>It's nearly 11 at night — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -14852,8 +15286,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F219" t="n">
-        <v>6</v>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -14902,7 +15338,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night � when should I run the washing machine?</t>
+          <t>It's nearly 11 at night — when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -14918,8 +15354,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F220" t="n">
-        <v>6</v>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -14984,8 +15422,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F221" t="n">
-        <v>4</v>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -15050,8 +15490,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F222" t="n">
-        <v>4</v>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -15116,8 +15558,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F223" t="n">
-        <v>4</v>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -15182,8 +15626,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F224" t="n">
-        <v>8</v>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -15248,8 +15694,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F225" t="n">
-        <v>8</v>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -15314,8 +15762,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F226" t="n">
-        <v>8</v>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -15364,7 +15814,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 � when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -15380,8 +15830,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F227" t="n">
-        <v>6</v>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -15430,7 +15882,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 � when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -15446,8 +15898,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F228" t="n">
-        <v>6</v>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -15496,7 +15950,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 � when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -15512,8 +15966,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F229" t="n">
-        <v>6</v>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -15578,8 +16034,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F230" t="n">
-        <v>35</v>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -15644,8 +16102,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F231" t="n">
-        <v>35</v>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -15710,8 +16170,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F232" t="n">
-        <v>35</v>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -15776,8 +16238,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F233" t="n">
-        <v>38</v>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -15842,8 +16306,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F234" t="n">
-        <v>38</v>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -15908,8 +16374,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F235" t="n">
-        <v>38</v>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -15974,8 +16442,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F236" t="n">
-        <v>32</v>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -16040,8 +16510,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F237" t="n">
-        <v>32</v>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -16106,8 +16578,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F238" t="n">
-        <v>32</v>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -16172,8 +16646,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F239" t="n">
-        <v>40</v>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -16238,8 +16714,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F240" t="n">
-        <v>40</v>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -16304,8 +16782,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F241" t="n">
-        <v>40</v>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -16370,8 +16850,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F242" t="n">
-        <v>7</v>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -16436,8 +16918,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F243" t="n">
-        <v>7</v>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -16502,8 +16986,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F244" t="n">
-        <v>7</v>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -16568,8 +17054,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F245" t="n">
-        <v>5</v>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -16634,8 +17122,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F246" t="n">
-        <v>5</v>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -16700,8 +17190,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F247" t="n">
-        <v>5</v>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -16766,8 +17258,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F248" t="n">
-        <v>9</v>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -16832,8 +17326,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F249" t="n">
-        <v>9</v>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -16898,8 +17394,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F250" t="n">
-        <v>9</v>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -16964,8 +17462,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F251" t="n">
-        <v>6</v>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -17030,8 +17530,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F252" t="n">
-        <v>6</v>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -17096,8 +17598,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F253" t="n">
-        <v>6</v>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -17162,8 +17666,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F254" t="n">
-        <v>8</v>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -17228,8 +17734,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F255" t="n">
-        <v>8</v>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -17294,8 +17802,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F256" t="n">
-        <v>8</v>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -17360,8 +17870,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F257" t="n">
-        <v>11</v>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -17426,8 +17938,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F258" t="n">
-        <v>11</v>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -17492,8 +18006,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F259" t="n">
-        <v>11</v>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -17558,8 +18074,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F260" t="n">
-        <v>5</v>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -17624,8 +18142,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F261" t="n">
-        <v>5</v>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -17690,8 +18210,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F262" t="n">
-        <v>5</v>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -17756,8 +18278,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F263" t="n">
-        <v>4</v>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -17822,8 +18346,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F264" t="n">
-        <v>4</v>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -17888,8 +18414,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F265" t="n">
-        <v>4</v>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -17954,8 +18482,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F266" t="n">
-        <v>9</v>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -18020,8 +18550,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F267" t="n">
-        <v>9</v>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -18086,8 +18618,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F268" t="n">
-        <v>9</v>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -18152,8 +18686,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F269" t="n">
-        <v>7</v>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -18218,8 +18754,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F270" t="n">
-        <v>7</v>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -18284,8 +18822,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F271" t="n">
-        <v>7</v>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -18350,8 +18890,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F272" t="n">
-        <v>6</v>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -18416,8 +18958,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F273" t="n">
-        <v>6</v>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -18482,8 +19026,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F274" t="n">
-        <v>6</v>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -18548,8 +19094,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F275" t="n">
-        <v>11</v>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -18614,8 +19162,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F276" t="n">
-        <v>11</v>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -18680,8 +19230,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F277" t="n">
-        <v>11</v>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
@@ -18746,8 +19298,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F278" t="n">
-        <v>3</v>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
@@ -18812,8 +19366,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F279" t="n">
-        <v>3</v>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
@@ -18878,8 +19434,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F280" t="n">
-        <v>3</v>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
@@ -18944,8 +19502,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F281" t="n">
-        <v>5</v>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
@@ -19010,8 +19570,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F282" t="n">
-        <v>5</v>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
@@ -19076,8 +19638,10 @@
           <t>washing_machine</t>
         </is>
       </c>
-      <c r="F283" t="n">
-        <v>5</v>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
@@ -19142,8 +19706,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F284" t="n">
-        <v>6</v>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G284" t="inlineStr">
         <is>
@@ -19208,8 +19774,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F285" t="n">
-        <v>6</v>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
@@ -19274,8 +19842,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F286" t="n">
-        <v>6</v>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G286" t="inlineStr">
         <is>
@@ -19340,8 +19910,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F287" t="n">
-        <v>4</v>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G287" t="inlineStr">
         <is>
@@ -19406,8 +19978,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F288" t="n">
-        <v>4</v>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G288" t="inlineStr">
         <is>
@@ -19472,8 +20046,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F289" t="n">
-        <v>4</v>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
@@ -19522,7 +20098,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -19538,8 +20114,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F290" t="n">
-        <v>7</v>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
@@ -19588,7 +20166,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -19604,8 +20182,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F291" t="n">
-        <v>7</v>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G291" t="inlineStr">
         <is>
@@ -19654,7 +20234,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon � when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -19670,8 +20250,10 @@
           <t>dryer</t>
         </is>
       </c>
-      <c r="F292" t="n">
-        <v>7</v>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
       </c>
       <c r="G292" t="inlineStr">
         <is>
@@ -19720,7 +20302,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -19736,8 +20318,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F293" t="n">
-        <v>10</v>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G293" t="inlineStr">
         <is>
@@ -19786,7 +20370,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -19802,8 +20386,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F294" t="n">
-        <v>10</v>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G294" t="inlineStr">
         <is>
@@ -19852,7 +20438,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>It's just got home � it's around 6 PM � and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -19868,8 +20454,10 @@
           <t>dishwasher</t>
         </is>
       </c>
-      <c r="F295" t="n">
-        <v>10</v>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
       <c r="G295" t="inlineStr">
         <is>
@@ -19931,11 +20519,13 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Dryer</t>
-        </is>
-      </c>
-      <c r="F296" t="n">
-        <v>9</v>
+          <t>dryer</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G296" t="inlineStr">
         <is>
@@ -19997,11 +20587,13 @@
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>Dryer</t>
-        </is>
-      </c>
-      <c r="F297" t="n">
-        <v>9</v>
+          <t>dryer</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G297" t="inlineStr">
         <is>
@@ -20063,11 +20655,13 @@
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>Dryer</t>
-        </is>
-      </c>
-      <c r="F298" t="n">
-        <v>9</v>
+          <t>dryer</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
       </c>
       <c r="G298" t="inlineStr">
         <is>
@@ -20129,11 +20723,13 @@
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>Dishwasher</t>
-        </is>
-      </c>
-      <c r="F299" t="n">
-        <v>6</v>
+          <t>dishwasher</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G299" t="inlineStr">
         <is>
@@ -20195,11 +20791,13 @@
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>Dishwasher</t>
-        </is>
-      </c>
-      <c r="F300" t="n">
-        <v>6</v>
+          <t>dishwasher</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G300" t="inlineStr">
         <is>
@@ -20261,11 +20859,13 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Dishwasher</t>
-        </is>
-      </c>
-      <c r="F301" t="n">
-        <v>6</v>
+          <t>dishwasher</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="G301" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Map Levittown->PECO and Quakertown->PPL; regenerate appliance ground truth
Appliance scenarios 92 (Levittown) and 95 (Quakertown) had cities absent
from CITY_TO_UTILITY, so their energy_cost silently fell back to 0 for all
alternatives (pre-existing). Added both to the PA city->utility map
(Levittown = PECO / lower Bucks; Quakertown = PPL / upper Bucks) and re-ran
the appliance calculator.

Now both scenarios get real TOU energy costs and differentiated rankings
(e.g. Levittown 8AM off-peak ranks #1, 2PM peak ranks #3). 0 unmapped-city
errors; MAVT integrity verified (0 violations across 100 scenarios).
Neither scenario is in the RAG partition, so RAG/ChromaDB are unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_appliance.xlsx
+++ b/Ground Truth/ground_truth_appliance.xlsx
@@ -19320,7 +19320,7 @@
         </is>
       </c>
       <c r="K278" t="n">
-        <v>10</v>
+        <v>9.57</v>
       </c>
       <c r="L278" t="n">
         <v>8.119999999999999</v>
@@ -19332,13 +19332,13 @@
         <v>10</v>
       </c>
       <c r="O278" t="n">
-        <v>9.341999999999999</v>
+        <v>9.212999999999999</v>
       </c>
       <c r="P278" t="n">
         <v>1</v>
       </c>
       <c r="Q278" t="n">
-        <v>0</v>
+        <v>0.0646</v>
       </c>
       <c r="R278" t="n">
         <v>0.885</v>
@@ -19388,7 +19388,7 @@
         </is>
       </c>
       <c r="K279" t="n">
-        <v>10</v>
+        <v>7.69</v>
       </c>
       <c r="L279" t="n">
         <v>8.119999999999999</v>
@@ -19400,13 +19400,13 @@
         <v>6.21</v>
       </c>
       <c r="O279" t="n">
-        <v>8.259499999999999</v>
+        <v>7.566499999999999</v>
       </c>
       <c r="P279" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q279" t="n">
-        <v>0</v>
+        <v>0.272</v>
       </c>
       <c r="R279" t="n">
         <v>0.885</v>
@@ -19456,7 +19456,7 @@
         </is>
       </c>
       <c r="K280" t="n">
-        <v>10</v>
+        <v>9.57</v>
       </c>
       <c r="L280" t="n">
         <v>8.279999999999999</v>
@@ -19468,13 +19468,13 @@
         <v>3.63</v>
       </c>
       <c r="O280" t="n">
-        <v>7.7005</v>
+        <v>7.5715</v>
       </c>
       <c r="P280" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q280" t="n">
-        <v>0</v>
+        <v>0.0646</v>
       </c>
       <c r="R280" t="n">
         <v>0.83</v>
@@ -19932,7 +19932,7 @@
         </is>
       </c>
       <c r="K287" t="n">
-        <v>10</v>
+        <v>9.16</v>
       </c>
       <c r="L287" t="n">
         <v>7.35</v>
@@ -19944,13 +19944,13 @@
         <v>10</v>
       </c>
       <c r="O287" t="n">
-        <v>9.0725</v>
+        <v>8.820499999999999</v>
       </c>
       <c r="P287" t="n">
         <v>1</v>
       </c>
       <c r="Q287" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="R287" t="n">
         <v>1.145</v>
@@ -20000,7 +20000,7 @@
         </is>
       </c>
       <c r="K288" t="n">
-        <v>10</v>
+        <v>8.76</v>
       </c>
       <c r="L288" t="n">
         <v>7.35</v>
@@ -20012,13 +20012,13 @@
         <v>7.15</v>
       </c>
       <c r="O288" t="n">
-        <v>8.291</v>
+        <v>7.919</v>
       </c>
       <c r="P288" t="n">
         <v>2</v>
       </c>
       <c r="Q288" t="n">
-        <v>0</v>
+        <v>0.154</v>
       </c>
       <c r="R288" t="n">
         <v>1.145</v>
@@ -20068,7 +20068,7 @@
         </is>
       </c>
       <c r="K289" t="n">
-        <v>10</v>
+        <v>9.16</v>
       </c>
       <c r="L289" t="n">
         <v>7.35</v>
@@ -20080,13 +20080,13 @@
         <v>2.7</v>
       </c>
       <c r="O289" t="n">
-        <v>7.0835</v>
+        <v>6.831499999999999</v>
       </c>
       <c r="P289" t="n">
         <v>3</v>
       </c>
       <c r="Q289" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="R289" t="n">
         <v>1.145</v>

</xml_diff>

<commit_message>
Refactor code structure for improved readability and maintainability
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_appliance.xlsx
+++ b/Ground Truth/ground_truth_appliance.xlsx
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>It's just past 5 PM — when should I run the dryer?</t>
+          <t>It's just past 5 PM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>It's just past 5 PM — when should I run the dryer?</t>
+          <t>It's just past 5 PM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1466,7 +1466,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>It's just past 5 PM — when should I run the dryer?</t>
+          <t>It's just past 5 PM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2350,7 +2350,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>It's around 7 in the evening — when should I run the dishwasher?</t>
+          <t>It's around 7 in the evening, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>It's around 7 in the evening — when should I run the dishwasher?</t>
+          <t>It's around 7 in the evening, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>It's around 7 in the evening — when should I run the dishwasher?</t>
+          <t>It's around 7 in the evening, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>It's getting close to midnight — when should I run the washing machine?</t>
+          <t>It's getting close to midnight, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>It's getting close to midnight — when should I run the washing machine?</t>
+          <t>It's getting close to midnight, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>It's getting close to midnight — when should I run the washing machine?</t>
+          <t>It's getting close to midnight, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3778,7 +3778,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>It's just past 5 PM — when should I run the washer?</t>
+          <t>It's just past 5 PM, when should I run the washer?</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -3846,7 +3846,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>It's just past 5 PM — when should I run the washer?</t>
+          <t>It's just past 5 PM, when should I run the washer?</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>It's just past 5 PM — when should I run the washer?</t>
+          <t>It's just past 5 PM, when should I run the washer?</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5410,7 +5410,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>It's past 1 in the morning — when should I run the dryer?</t>
+          <t>It's past 1 in the morning, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>It's past 1 in the morning — when should I run the dryer?</t>
+          <t>It's past 1 in the morning, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>It's past 1 in the morning — when should I run the dryer?</t>
+          <t>It's past 1 in the morning, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -6226,7 +6226,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>It's just past midnight — when should I run the dishwasher?</t>
+          <t>It's just past midnight, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -6294,7 +6294,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>It's just past midnight — when should I run the dishwasher?</t>
+          <t>It's just past midnight, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -6362,7 +6362,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>It's just past midnight — when should I run the dishwasher?</t>
+          <t>It's just past midnight, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>It's around 8 at night — when should I run the dishwasher?</t>
+          <t>It's around 8 at night, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -7314,7 +7314,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>It's around 8 at night — when should I run the dishwasher?</t>
+          <t>It's around 8 at night, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>It's around 8 at night — when should I run the dishwasher?</t>
+          <t>It's around 8 at night, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -8674,7 +8674,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>It's just past 9 AM — when should I run the dryer?</t>
+          <t>It's just past 9 AM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -8742,7 +8742,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>It's just past 9 AM — when should I run the dryer?</t>
+          <t>It's just past 9 AM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>It's just past 9 AM — when should I run the dryer?</t>
+          <t>It's just past 9 AM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -10510,7 +10510,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>It's just past 9 AM — when should I run the dryer?</t>
+          <t>It's just past 9 AM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -10578,7 +10578,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>It's just past 9 AM — when should I run the dryer?</t>
+          <t>It's just past 9 AM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -10646,7 +10646,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>It's just past 9 AM — when should I run the dryer?</t>
+          <t>It's just past 9 AM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -11326,7 +11326,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening — when should I run the washing machine?</t>
+          <t>It's around 5 in the evening, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -11394,7 +11394,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening — when should I run the washing machine?</t>
+          <t>It's around 5 in the evening, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>It's around 5 in the evening — when should I run the washing machine?</t>
+          <t>It's around 5 in the evening, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -11734,7 +11734,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>It's just past 7 PM — when should I run the dryer?</t>
+          <t>It's just past 7 PM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -11802,7 +11802,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>It's just past 7 PM — when should I run the dryer?</t>
+          <t>It's just past 7 PM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>It's just past 7 PM — when should I run the dryer?</t>
+          <t>It's just past 7 PM, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -12346,7 +12346,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late, just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -12414,7 +12414,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late, just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -12482,7 +12482,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>It's late — just past 10 PM and I need to run the dryer. When should I start it?</t>
+          <t>It's late, just past 10 PM and I need to run the dryer. When should I start it?</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -12958,7 +12958,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>It's getting close to midnight — when should I run the washing machine?</t>
+          <t>It's getting close to midnight, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -13026,7 +13026,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>It's getting close to midnight — when should I run the washing machine?</t>
+          <t>It's getting close to midnight, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -13094,7 +13094,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>It's getting close to midnight — when should I run the washing machine?</t>
+          <t>It's getting close to midnight, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -13570,7 +13570,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>It's just after 8 AM — when should I run the dishwasher?</t>
+          <t>It's just after 8 AM, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -13638,7 +13638,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>It's just after 8 AM — when should I run the dishwasher?</t>
+          <t>It's just after 8 AM, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -13706,7 +13706,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>It's just after 8 AM — when should I run the dishwasher?</t>
+          <t>It's just after 8 AM, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -15202,7 +15202,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night — when should I run the washing machine?</t>
+          <t>It's nearly 11 at night, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -15270,7 +15270,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night — when should I run the washing machine?</t>
+          <t>It's nearly 11 at night, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -15338,7 +15338,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>It's nearly 11 at night — when should I run the washing machine?</t>
+          <t>It's nearly 11 at night, when should I run the washing machine?</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -15814,7 +15814,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -15882,7 +15882,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -15950,7 +15950,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>It's late afternoon, just past 3 — when should I run the dishwasher?</t>
+          <t>It's late afternoon, just past 3, when should I run the dishwasher?</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -20098,7 +20098,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -20166,7 +20166,7 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -20234,7 +20234,7 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>It's around 2 in the afternoon — when should I run the dryer?</t>
+          <t>It's around 2 in the afternoon, when should I run the dryer?</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -20302,7 +20302,7 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home, it's around 6 PM, and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -20370,7 +20370,7 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home, it's around 6 PM, and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
@@ -20438,7 +20438,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>I've just got home — it's around 6 PM — and I need to run the dishwasher. When should I start it?</t>
+          <t>I've just got home, it's around 6 PM, and I need to run the dishwasher. When should I start it?</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">

</xml_diff>

<commit_message>
ran ground truth, synced Rag, and ran buildRAG
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_appliance.xlsx
+++ b/Ground Truth/ground_truth_appliance.xlsx
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="K2" t="n">
-        <v>9.48</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L2" t="n">
         <v>9.34</v>
@@ -564,13 +564,13 @@
         <v>10</v>
       </c>
       <c r="O2" t="n">
-        <v>9.613</v>
+        <v>9.606999999999999</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0743</v>
+        <v>0.0774</v>
       </c>
       <c r="R2" t="n">
         <v>0.468</v>
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>9.880000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L3" t="n">
         <v>9.34</v>
@@ -632,13 +632,13 @@
         <v>4.97</v>
       </c>
       <c r="O3" t="n">
-        <v>8.2545</v>
+        <v>8.230499999999999</v>
       </c>
       <c r="P3" t="n">
         <v>2</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0302</v>
+        <v>0.0396</v>
       </c>
       <c r="R3" t="n">
         <v>0.468</v>
@@ -688,7 +688,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>9.880000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L4" t="n">
         <v>9.43</v>
@@ -700,13 +700,13 @@
         <v>4.31</v>
       </c>
       <c r="O4" t="n">
-        <v>7.582999999999999</v>
+        <v>7.558999999999998</v>
       </c>
       <c r="P4" t="n">
         <v>3</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.0302</v>
+        <v>0.0396</v>
       </c>
       <c r="R4" t="n">
         <v>0.439</v>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>5.37</v>
+        <v>5.17</v>
       </c>
       <c r="L5" t="n">
         <v>0.92</v>
@@ -768,13 +768,13 @@
         <v>10</v>
       </c>
       <c r="O5" t="n">
-        <v>5.433</v>
+        <v>5.373</v>
       </c>
       <c r="P5" t="n">
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>0.528</v>
+        <v>0.5504</v>
       </c>
       <c r="R5" t="n">
         <v>3.331</v>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="K6" t="n">
-        <v>8.210000000000001</v>
+        <v>7.6</v>
       </c>
       <c r="L6" t="n">
         <v>1.53</v>
@@ -836,13 +836,13 @@
         <v>5.67</v>
       </c>
       <c r="O6" t="n">
-        <v>4.869</v>
+        <v>4.686</v>
       </c>
       <c r="P6" t="n">
         <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.2144</v>
+        <v>0.2816</v>
       </c>
       <c r="R6" t="n">
         <v>3.123</v>
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>5.37</v>
+        <v>5.17</v>
       </c>
       <c r="L7" t="n">
         <v>0.92</v>
@@ -904,13 +904,13 @@
         <v>6.04</v>
       </c>
       <c r="O7" t="n">
-        <v>4.297</v>
+        <v>4.237</v>
       </c>
       <c r="P7" t="n">
         <v>3</v>
       </c>
       <c r="Q7" t="n">
-        <v>0.528</v>
+        <v>0.5504</v>
       </c>
       <c r="R7" t="n">
         <v>3.331</v>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="K8" t="n">
-        <v>9.33</v>
+        <v>9.08</v>
       </c>
       <c r="L8" t="n">
         <v>6.84</v>
@@ -972,13 +972,13 @@
         <v>9.25</v>
       </c>
       <c r="O8" t="n">
-        <v>8.580499999999999</v>
+        <v>8.5055</v>
       </c>
       <c r="P8" t="n">
         <v>1</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.0905</v>
+        <v>0.1188</v>
       </c>
       <c r="R8" t="n">
         <v>1.318</v>
@@ -1028,7 +1028,7 @@
         </is>
       </c>
       <c r="K9" t="n">
-        <v>8.130000000000001</v>
+        <v>8.050000000000001</v>
       </c>
       <c r="L9" t="n">
         <v>6.58</v>
@@ -1040,13 +1040,13 @@
         <v>4.64</v>
       </c>
       <c r="O9" t="n">
-        <v>6.584</v>
+        <v>6.56</v>
       </c>
       <c r="P9" t="n">
         <v>3</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2228</v>
+        <v>0.2322</v>
       </c>
       <c r="R9" t="n">
         <v>1.405</v>
@@ -1096,7 +1096,7 @@
         </is>
       </c>
       <c r="K10" t="n">
-        <v>9.33</v>
+        <v>9.08</v>
       </c>
       <c r="L10" t="n">
         <v>6.58</v>
@@ -1108,13 +1108,13 @@
         <v>4.64</v>
       </c>
       <c r="O10" t="n">
-        <v>6.944</v>
+        <v>6.868999999999999</v>
       </c>
       <c r="P10" t="n">
         <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.0905</v>
+        <v>0.1188</v>
       </c>
       <c r="R10" t="n">
         <v>1.405</v>
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="K11" t="n">
-        <v>9.98</v>
+        <v>9.94</v>
       </c>
       <c r="L11" t="n">
         <v>9.859999999999999</v>
@@ -1176,13 +1176,13 @@
         <v>10</v>
       </c>
       <c r="O11" t="n">
-        <v>9.945</v>
+        <v>9.933</v>
       </c>
       <c r="P11" t="n">
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.0188</v>
+        <v>0.0246</v>
       </c>
       <c r="R11" t="n">
         <v>0.291</v>
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>9.74</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="L12" t="n">
         <v>9.859999999999999</v>
@@ -1244,13 +1244,13 @@
         <v>6.78</v>
       </c>
       <c r="O12" t="n">
-        <v>8.972</v>
+        <v>8.965999999999999</v>
       </c>
       <c r="P12" t="n">
         <v>2</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.0462</v>
+        <v>0.0482</v>
       </c>
       <c r="R12" t="n">
         <v>0.291</v>
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>9.98</v>
+        <v>9.94</v>
       </c>
       <c r="L13" t="n">
         <v>9.859999999999999</v>
@@ -1312,13 +1312,13 @@
         <v>1.51</v>
       </c>
       <c r="O13" t="n">
-        <v>7.1415</v>
+        <v>7.129499999999999</v>
       </c>
       <c r="P13" t="n">
         <v>3</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.0188</v>
+        <v>0.0246</v>
       </c>
       <c r="R13" t="n">
         <v>0.291</v>
@@ -1368,7 +1368,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>4.92</v>
+        <v>4.7</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
@@ -1380,13 +1380,13 @@
         <v>10</v>
       </c>
       <c r="O14" t="n">
-        <v>4.976</v>
+        <v>4.91</v>
       </c>
       <c r="P14" t="n">
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.5775</v>
+        <v>0.602</v>
       </c>
       <c r="R14" t="n">
         <v>3.643</v>
@@ -1436,7 +1436,7 @@
         </is>
       </c>
       <c r="K15" t="n">
-        <v>4.92</v>
+        <v>4.7</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -1448,13 +1448,13 @@
         <v>7.82</v>
       </c>
       <c r="O15" t="n">
-        <v>4.369</v>
+        <v>4.303</v>
       </c>
       <c r="P15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0.5775</v>
+        <v>0.602</v>
       </c>
       <c r="R15" t="n">
         <v>3.643</v>
@@ -1504,7 +1504,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>8.029999999999999</v>
+        <v>7.37</v>
       </c>
       <c r="L16" t="n">
         <v>0.67</v>
@@ -1516,13 +1516,13 @@
         <v>5.19</v>
       </c>
       <c r="O16" t="n">
-        <v>4.468</v>
+        <v>4.27</v>
       </c>
       <c r="P16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.2345</v>
+        <v>0.308</v>
       </c>
       <c r="R16" t="n">
         <v>3.416</v>
@@ -1572,7 +1572,7 @@
         </is>
       </c>
       <c r="K17" t="n">
-        <v>9.76</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="L17" t="n">
         <v>8.85</v>
@@ -1584,13 +1584,13 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O17" t="n">
-        <v>8.858999999999998</v>
+        <v>8.822999999999999</v>
       </c>
       <c r="P17" t="n">
         <v>1</v>
       </c>
       <c r="Q17" t="n">
-        <v>0.0436</v>
+        <v>0.0572</v>
       </c>
       <c r="R17" t="n">
         <v>0.634</v>
@@ -1640,7 +1640,7 @@
         </is>
       </c>
       <c r="K18" t="n">
-        <v>9.76</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="L18" t="n">
         <v>8.73</v>
@@ -1652,13 +1652,13 @@
         <v>4.64</v>
       </c>
       <c r="O18" t="n">
-        <v>7.725499999999999</v>
+        <v>7.6895</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
       </c>
       <c r="Q18" t="n">
-        <v>0.0436</v>
+        <v>0.0572</v>
       </c>
       <c r="R18" t="n">
         <v>0.677</v>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="K19" t="n">
-        <v>9.18</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="L19" t="n">
         <v>8.73</v>
@@ -1720,13 +1720,13 @@
         <v>2.03</v>
       </c>
       <c r="O19" t="n">
-        <v>6.902</v>
+        <v>6.89</v>
       </c>
       <c r="P19" t="n">
         <v>3</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.1073</v>
+        <v>0.1118</v>
       </c>
       <c r="R19" t="n">
         <v>0.677</v>
@@ -1776,7 +1776,7 @@
         </is>
       </c>
       <c r="K20" t="n">
-        <v>5.97</v>
+        <v>5.79</v>
       </c>
       <c r="L20" t="n">
         <v>2.14</v>
@@ -1788,13 +1788,13 @@
         <v>10</v>
       </c>
       <c r="O20" t="n">
-        <v>6.04</v>
+        <v>5.986</v>
       </c>
       <c r="P20" t="n">
         <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.462</v>
+        <v>0.4816</v>
       </c>
       <c r="R20" t="n">
         <v>2.915</v>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="K21" t="n">
-        <v>5.97</v>
+        <v>5.79</v>
       </c>
       <c r="L21" t="n">
         <v>2.14</v>
@@ -1856,13 +1856,13 @@
         <v>6.04</v>
       </c>
       <c r="O21" t="n">
-        <v>4.904</v>
+        <v>4.85</v>
       </c>
       <c r="P21" t="n">
         <v>2</v>
       </c>
       <c r="Q21" t="n">
-        <v>0.462</v>
+        <v>0.4816</v>
       </c>
       <c r="R21" t="n">
         <v>2.915</v>
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="K22" t="n">
-        <v>8.449999999999999</v>
+        <v>7.92</v>
       </c>
       <c r="L22" t="n">
         <v>2.68</v>
@@ -1924,13 +1924,13 @@
         <v>3.11</v>
       </c>
       <c r="O22" t="n">
-        <v>4.611499999999999</v>
+        <v>4.452500000000001</v>
       </c>
       <c r="P22" t="n">
         <v>3</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.1876</v>
+        <v>0.2464</v>
       </c>
       <c r="R22" t="n">
         <v>2.733</v>
@@ -1980,7 +1980,7 @@
         </is>
       </c>
       <c r="K23" t="n">
-        <v>7.36</v>
+        <v>7.58</v>
       </c>
       <c r="L23" t="n">
         <v>6.43</v>
@@ -1992,13 +1992,13 @@
         <v>10</v>
       </c>
       <c r="O23" t="n">
-        <v>7.9585</v>
+        <v>8.0245</v>
       </c>
       <c r="P23" t="n">
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.308</v>
+        <v>0.2842</v>
       </c>
       <c r="R23" t="n">
         <v>1.457</v>
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="K24" t="n">
-        <v>7.36</v>
+        <v>7.58</v>
       </c>
       <c r="L24" t="n">
         <v>6.43</v>
@@ -2060,13 +2060,13 @@
         <v>9.199999999999999</v>
       </c>
       <c r="O24" t="n">
-        <v>7.7405</v>
+        <v>7.8065</v>
       </c>
       <c r="P24" t="n">
         <v>2</v>
       </c>
       <c r="Q24" t="n">
-        <v>0.308</v>
+        <v>0.2842</v>
       </c>
       <c r="R24" t="n">
         <v>1.457</v>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="K25" t="n">
-        <v>9.140000000000001</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="L25" t="n">
         <v>6.7</v>
@@ -2128,13 +2128,13 @@
         <v>2.89</v>
       </c>
       <c r="O25" t="n">
-        <v>6.666499999999999</v>
+        <v>6.5915</v>
       </c>
       <c r="P25" t="n">
         <v>3</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.112</v>
+        <v>0.14</v>
       </c>
       <c r="R25" t="n">
         <v>1.366</v>
@@ -2796,7 +2796,7 @@
         </is>
       </c>
       <c r="K35" t="n">
-        <v>9.050000000000001</v>
+        <v>9.06</v>
       </c>
       <c r="L35" t="n">
         <v>9.550000000000001</v>
@@ -2808,7 +2808,7 @@
         <v>10</v>
       </c>
       <c r="O35" t="n">
-        <v>9.557500000000001</v>
+        <v>9.560500000000001</v>
       </c>
       <c r="P35" t="n">
         <v>1</v>
@@ -2864,7 +2864,7 @@
         </is>
       </c>
       <c r="K36" t="n">
-        <v>9.890000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="L36" t="n">
         <v>9.550000000000001</v>
@@ -2876,7 +2876,7 @@
         <v>3.11</v>
       </c>
       <c r="O36" t="n">
-        <v>7.298</v>
+        <v>7.301</v>
       </c>
       <c r="P36" t="n">
         <v>2</v>
@@ -2932,7 +2932,7 @@
         </is>
       </c>
       <c r="K37" t="n">
-        <v>9.890000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="L37" t="n">
         <v>9.630000000000001</v>
@@ -2944,7 +2944,7 @@
         <v>1.51</v>
       </c>
       <c r="O37" t="n">
-        <v>6.752</v>
+        <v>6.755</v>
       </c>
       <c r="P37" t="n">
         <v>3</v>
@@ -3000,7 +3000,7 @@
         </is>
       </c>
       <c r="K38" t="n">
-        <v>7.74</v>
+        <v>7.75</v>
       </c>
       <c r="L38" t="n">
         <v>0.67</v>
@@ -3012,7 +3012,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O38" t="n">
-        <v>5.484</v>
+        <v>5.487</v>
       </c>
       <c r="P38" t="n">
         <v>1</v>
@@ -3136,7 +3136,7 @@
         </is>
       </c>
       <c r="K40" t="n">
-        <v>7.74</v>
+        <v>7.75</v>
       </c>
       <c r="L40" t="n">
         <v>0.67</v>
@@ -3148,7 +3148,7 @@
         <v>7.37</v>
       </c>
       <c r="O40" t="n">
-        <v>5.062</v>
+        <v>5.065</v>
       </c>
       <c r="P40" t="n">
         <v>2</v>
@@ -3544,7 +3544,7 @@
         </is>
       </c>
       <c r="K46" t="n">
-        <v>9.529999999999999</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="L46" t="n">
         <v>7.81</v>
@@ -3556,13 +3556,13 @@
         <v>5.05</v>
       </c>
       <c r="O46" t="n">
-        <v>7.814</v>
+        <v>7.763</v>
       </c>
       <c r="P46" t="n">
         <v>3</v>
       </c>
       <c r="Q46" t="n">
-        <v>0.0684</v>
+        <v>0.0883</v>
       </c>
       <c r="R46" t="n">
         <v>0.989</v>
@@ -3952,7 +3952,7 @@
         </is>
       </c>
       <c r="K52" t="n">
-        <v>9.91</v>
+        <v>9.84</v>
       </c>
       <c r="L52" t="n">
         <v>9.550000000000001</v>
@@ -3964,13 +3964,13 @@
         <v>6.78</v>
       </c>
       <c r="O52" t="n">
-        <v>8.9145</v>
+        <v>8.8935</v>
       </c>
       <c r="P52" t="n">
         <v>3</v>
       </c>
       <c r="Q52" t="n">
-        <v>0.0274</v>
+        <v>0.0353</v>
       </c>
       <c r="R52" t="n">
         <v>0.396</v>
@@ -4020,7 +4020,7 @@
         </is>
       </c>
       <c r="K53" t="n">
-        <v>4.28</v>
+        <v>4.29</v>
       </c>
       <c r="L53" t="n">
         <v>0</v>
@@ -4032,7 +4032,7 @@
         <v>10</v>
       </c>
       <c r="O53" t="n">
-        <v>4.784</v>
+        <v>4.787</v>
       </c>
       <c r="P53" t="n">
         <v>1</v>
@@ -4088,7 +4088,7 @@
         </is>
       </c>
       <c r="K54" t="n">
-        <v>7.87</v>
+        <v>7.21</v>
       </c>
       <c r="L54" t="n">
         <v>0.67</v>
@@ -4100,13 +4100,13 @@
         <v>1.51</v>
       </c>
       <c r="O54" t="n">
-        <v>3.588</v>
+        <v>3.39</v>
       </c>
       <c r="P54" t="n">
         <v>3</v>
       </c>
       <c r="Q54" t="n">
-        <v>0.252</v>
+        <v>0.3255</v>
       </c>
       <c r="R54" t="n">
         <v>3.416</v>
@@ -4156,7 +4156,7 @@
         </is>
       </c>
       <c r="K55" t="n">
-        <v>7.87</v>
+        <v>7.21</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
@@ -4168,13 +4168,13 @@
         <v>4.31</v>
       </c>
       <c r="O55" t="n">
-        <v>4.0535</v>
+        <v>3.8555</v>
       </c>
       <c r="P55" t="n">
         <v>2</v>
       </c>
       <c r="Q55" t="n">
-        <v>0.252</v>
+        <v>0.3255</v>
       </c>
       <c r="R55" t="n">
         <v>3.643</v>
@@ -4224,7 +4224,7 @@
         </is>
       </c>
       <c r="K56" t="n">
-        <v>9.68</v>
+        <v>9.69</v>
       </c>
       <c r="L56" t="n">
         <v>9.859999999999999</v>
@@ -4236,7 +4236,7 @@
         <v>10</v>
       </c>
       <c r="O56" t="n">
-        <v>9.855</v>
+        <v>9.857999999999999</v>
       </c>
       <c r="P56" t="n">
         <v>1</v>
@@ -4292,7 +4292,7 @@
         </is>
       </c>
       <c r="K57" t="n">
-        <v>9.970000000000001</v>
+        <v>9.92</v>
       </c>
       <c r="L57" t="n">
         <v>9.859999999999999</v>
@@ -4304,13 +4304,13 @@
         <v>6.78</v>
       </c>
       <c r="O57" t="n">
-        <v>9.041</v>
+        <v>9.026</v>
       </c>
       <c r="P57" t="n">
         <v>2</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.0202</v>
+        <v>0.026</v>
       </c>
       <c r="R57" t="n">
         <v>0.291</v>
@@ -4360,7 +4360,7 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>9.970000000000001</v>
+        <v>9.92</v>
       </c>
       <c r="L58" t="n">
         <v>9.859999999999999</v>
@@ -4372,13 +4372,13 @@
         <v>6.21</v>
       </c>
       <c r="O58" t="n">
-        <v>8.859500000000001</v>
+        <v>8.8445</v>
       </c>
       <c r="P58" t="n">
         <v>3</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.0202</v>
+        <v>0.026</v>
       </c>
       <c r="R58" t="n">
         <v>0.291</v>
@@ -4428,7 +4428,7 @@
         </is>
       </c>
       <c r="K59" t="n">
-        <v>8.26</v>
+        <v>8.41</v>
       </c>
       <c r="L59" t="n">
         <v>7.81</v>
@@ -4440,13 +4440,13 @@
         <v>10</v>
       </c>
       <c r="O59" t="n">
-        <v>8.711499999999999</v>
+        <v>8.756499999999999</v>
       </c>
       <c r="P59" t="n">
         <v>1</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.209</v>
+        <v>0.1928</v>
       </c>
       <c r="R59" t="n">
         <v>0.989</v>
@@ -4496,7 +4496,7 @@
         </is>
       </c>
       <c r="K60" t="n">
-        <v>9.470000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L60" t="n">
         <v>7.99</v>
@@ -4508,13 +4508,13 @@
         <v>2.86</v>
       </c>
       <c r="O60" t="n">
-        <v>7.396500000000001</v>
+        <v>7.3455</v>
       </c>
       <c r="P60" t="n">
         <v>3</v>
       </c>
       <c r="Q60" t="n">
-        <v>0.076</v>
+        <v>0.095</v>
       </c>
       <c r="R60" t="n">
         <v>0.927</v>
@@ -4564,7 +4564,7 @@
         </is>
       </c>
       <c r="K61" t="n">
-        <v>8.26</v>
+        <v>8.41</v>
       </c>
       <c r="L61" t="n">
         <v>7.81</v>
@@ -4576,13 +4576,13 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O61" t="n">
-        <v>8.296999999999999</v>
+        <v>8.342000000000001</v>
       </c>
       <c r="P61" t="n">
         <v>2</v>
       </c>
       <c r="Q61" t="n">
-        <v>0.209</v>
+        <v>0.1928</v>
       </c>
       <c r="R61" t="n">
         <v>0.989</v>
@@ -4632,7 +4632,7 @@
         </is>
       </c>
       <c r="K62" t="n">
-        <v>9.4</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L62" t="n">
         <v>9.550000000000001</v>
@@ -4644,13 +4644,13 @@
         <v>10</v>
       </c>
       <c r="O62" t="n">
-        <v>9.6625</v>
+        <v>9.6805</v>
       </c>
       <c r="P62" t="n">
         <v>1</v>
       </c>
       <c r="Q62" t="n">
-        <v>0.08359999999999999</v>
+        <v>0.0771</v>
       </c>
       <c r="R62" t="n">
         <v>0.396</v>
@@ -4700,7 +4700,7 @@
         </is>
       </c>
       <c r="K63" t="n">
-        <v>9.4</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L63" t="n">
         <v>9.550000000000001</v>
@@ -4712,13 +4712,13 @@
         <v>6.21</v>
       </c>
       <c r="O63" t="n">
-        <v>8.58</v>
+        <v>8.598000000000001</v>
       </c>
       <c r="P63" t="n">
         <v>2</v>
       </c>
       <c r="Q63" t="n">
-        <v>0.08359999999999999</v>
+        <v>0.0771</v>
       </c>
       <c r="R63" t="n">
         <v>0.396</v>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
       <c r="K64" t="n">
-        <v>9.880000000000001</v>
+        <v>9.81</v>
       </c>
       <c r="L64" t="n">
         <v>9.630000000000001</v>
@@ -4780,13 +4780,13 @@
         <v>3.36</v>
       </c>
       <c r="O64" t="n">
-        <v>7.9245</v>
+        <v>7.903500000000001</v>
       </c>
       <c r="P64" t="n">
         <v>3</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.0304</v>
+        <v>0.038</v>
       </c>
       <c r="R64" t="n">
         <v>0.371</v>
@@ -4836,7 +4836,7 @@
         </is>
       </c>
       <c r="K65" t="n">
-        <v>3.17</v>
+        <v>3.71</v>
       </c>
       <c r="L65" t="n">
         <v>0</v>
@@ -4848,13 +4848,13 @@
         <v>10</v>
       </c>
       <c r="O65" t="n">
-        <v>4.451000000000001</v>
+        <v>4.613</v>
       </c>
       <c r="P65" t="n">
         <v>1</v>
       </c>
       <c r="Q65" t="n">
-        <v>0.77</v>
+        <v>0.7105</v>
       </c>
       <c r="R65" t="n">
         <v>3.643</v>
@@ -4904,7 +4904,7 @@
         </is>
       </c>
       <c r="K66" t="n">
-        <v>7.62</v>
+        <v>6.98</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -4916,13 +4916,13 @@
         <v>4.36</v>
       </c>
       <c r="O66" t="n">
-        <v>3.828</v>
+        <v>3.636</v>
       </c>
       <c r="P66" t="n">
         <v>2</v>
       </c>
       <c r="Q66" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="R66" t="n">
         <v>3.643</v>
@@ -4972,7 +4972,7 @@
         </is>
       </c>
       <c r="K67" t="n">
-        <v>7.62</v>
+        <v>6.98</v>
       </c>
       <c r="L67" t="n">
         <v>0.67</v>
@@ -4984,13 +4984,13 @@
         <v>1.51</v>
       </c>
       <c r="O67" t="n">
-        <v>3.243</v>
+        <v>3.051</v>
       </c>
       <c r="P67" t="n">
         <v>3</v>
       </c>
       <c r="Q67" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="R67" t="n">
         <v>3.416</v>
@@ -5108,7 +5108,7 @@
         </is>
       </c>
       <c r="K69" t="n">
-        <v>7.74</v>
+        <v>7.75</v>
       </c>
       <c r="L69" t="n">
         <v>0.67</v>
@@ -5120,7 +5120,7 @@
         <v>3.72</v>
       </c>
       <c r="O69" t="n">
-        <v>3.7365</v>
+        <v>3.7395</v>
       </c>
       <c r="P69" t="n">
         <v>2</v>
@@ -5176,7 +5176,7 @@
         </is>
       </c>
       <c r="K70" t="n">
-        <v>7.74</v>
+        <v>7.75</v>
       </c>
       <c r="L70" t="n">
         <v>0</v>
@@ -5188,7 +5188,7 @@
         <v>4.86</v>
       </c>
       <c r="O70" t="n">
-        <v>4.309</v>
+        <v>4.311999999999999</v>
       </c>
       <c r="P70" t="n">
         <v>1</v>
@@ -5856,7 +5856,7 @@
         </is>
       </c>
       <c r="K80" t="n">
-        <v>7.74</v>
+        <v>7.75</v>
       </c>
       <c r="L80" t="n">
         <v>0.67</v>
@@ -5868,7 +5868,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O80" t="n">
-        <v>5.484</v>
+        <v>5.487</v>
       </c>
       <c r="P80" t="n">
         <v>1</v>
@@ -5924,7 +5924,7 @@
         </is>
       </c>
       <c r="K81" t="n">
-        <v>7.74</v>
+        <v>7.75</v>
       </c>
       <c r="L81" t="n">
         <v>0</v>
@@ -5936,7 +5936,7 @@
         <v>6.66</v>
       </c>
       <c r="O81" t="n">
-        <v>4.883</v>
+        <v>4.885999999999999</v>
       </c>
       <c r="P81" t="n">
         <v>2</v>
@@ -6060,7 +6060,7 @@
         </is>
       </c>
       <c r="K83" t="n">
-        <v>7.87</v>
+        <v>7.21</v>
       </c>
       <c r="L83" t="n">
         <v>0.67</v>
@@ -6072,13 +6072,13 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O83" t="n">
-        <v>5.429</v>
+        <v>5.231</v>
       </c>
       <c r="P83" t="n">
         <v>1</v>
       </c>
       <c r="Q83" t="n">
-        <v>0.252</v>
+        <v>0.3255</v>
       </c>
       <c r="R83" t="n">
         <v>3.416</v>
@@ -6128,7 +6128,7 @@
         </is>
       </c>
       <c r="K84" t="n">
-        <v>4.28</v>
+        <v>4.29</v>
       </c>
       <c r="L84" t="n">
         <v>0</v>
@@ -6140,7 +6140,7 @@
         <v>6.04</v>
       </c>
       <c r="O84" t="n">
-        <v>3.648</v>
+        <v>3.651</v>
       </c>
       <c r="P84" t="n">
         <v>2</v>
@@ -6196,7 +6196,7 @@
         </is>
       </c>
       <c r="K85" t="n">
-        <v>4.28</v>
+        <v>4.29</v>
       </c>
       <c r="L85" t="n">
         <v>0</v>
@@ -6208,7 +6208,7 @@
         <v>3.87</v>
       </c>
       <c r="O85" t="n">
-        <v>2.9705</v>
+        <v>2.9735</v>
       </c>
       <c r="P85" t="n">
         <v>3</v>
@@ -6536,7 +6536,7 @@
         </is>
       </c>
       <c r="K90" t="n">
-        <v>9.91</v>
+        <v>9.84</v>
       </c>
       <c r="L90" t="n">
         <v>9.550000000000001</v>
@@ -6548,13 +6548,13 @@
         <v>5.19</v>
       </c>
       <c r="O90" t="n">
-        <v>8.295999999999999</v>
+        <v>8.275</v>
       </c>
       <c r="P90" t="n">
         <v>2</v>
       </c>
       <c r="Q90" t="n">
-        <v>0.0274</v>
+        <v>0.0353</v>
       </c>
       <c r="R90" t="n">
         <v>0.396</v>
@@ -6604,7 +6604,7 @@
         </is>
       </c>
       <c r="K91" t="n">
-        <v>9.91</v>
+        <v>9.84</v>
       </c>
       <c r="L91" t="n">
         <v>9.630000000000001</v>
@@ -6616,13 +6616,13 @@
         <v>4.36</v>
       </c>
       <c r="O91" t="n">
-        <v>7.8535</v>
+        <v>7.8325</v>
       </c>
       <c r="P91" t="n">
         <v>3</v>
       </c>
       <c r="Q91" t="n">
-        <v>0.0274</v>
+        <v>0.0353</v>
       </c>
       <c r="R91" t="n">
         <v>0.371</v>
@@ -6672,7 +6672,7 @@
         </is>
       </c>
       <c r="K92" t="n">
-        <v>3.17</v>
+        <v>3.71</v>
       </c>
       <c r="L92" t="n">
         <v>0</v>
@@ -6684,13 +6684,13 @@
         <v>10</v>
       </c>
       <c r="O92" t="n">
-        <v>4.451000000000001</v>
+        <v>4.613</v>
       </c>
       <c r="P92" t="n">
         <v>1</v>
       </c>
       <c r="Q92" t="n">
-        <v>0.77</v>
+        <v>0.7105</v>
       </c>
       <c r="R92" t="n">
         <v>3.643</v>
@@ -6740,7 +6740,7 @@
         </is>
       </c>
       <c r="K93" t="n">
-        <v>7.62</v>
+        <v>6.98</v>
       </c>
       <c r="L93" t="n">
         <v>0.67</v>
@@ -6752,13 +6752,13 @@
         <v>4.08</v>
       </c>
       <c r="O93" t="n">
-        <v>3.9885</v>
+        <v>3.7965</v>
       </c>
       <c r="P93" t="n">
         <v>2</v>
       </c>
       <c r="Q93" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="R93" t="n">
         <v>3.416</v>
@@ -6808,7 +6808,7 @@
         </is>
       </c>
       <c r="K94" t="n">
-        <v>7.62</v>
+        <v>6.98</v>
       </c>
       <c r="L94" t="n">
         <v>0.67</v>
@@ -6820,13 +6820,13 @@
         <v>1.86</v>
       </c>
       <c r="O94" t="n">
-        <v>3.4715</v>
+        <v>3.2795</v>
       </c>
       <c r="P94" t="n">
         <v>3</v>
       </c>
       <c r="Q94" t="n">
-        <v>0.28</v>
+        <v>0.35</v>
       </c>
       <c r="R94" t="n">
         <v>3.416</v>
@@ -6876,7 +6876,7 @@
         </is>
       </c>
       <c r="K95" t="n">
-        <v>5.17</v>
+        <v>5.56</v>
       </c>
       <c r="L95" t="n">
         <v>3.06</v>
@@ -6888,13 +6888,13 @@
         <v>10</v>
       </c>
       <c r="O95" t="n">
-        <v>6.122</v>
+        <v>6.239</v>
       </c>
       <c r="P95" t="n">
         <v>1</v>
       </c>
       <c r="Q95" t="n">
-        <v>0.55</v>
+        <v>0.5075</v>
       </c>
       <c r="R95" t="n">
         <v>2.603</v>
@@ -6944,7 +6944,7 @@
         </is>
       </c>
       <c r="K96" t="n">
-        <v>8.34</v>
+        <v>7.89</v>
       </c>
       <c r="L96" t="n">
         <v>3.54</v>
@@ -6956,13 +6956,13 @@
         <v>1.51</v>
       </c>
       <c r="O96" t="n">
-        <v>4.273499999999999</v>
+        <v>4.1385</v>
       </c>
       <c r="P96" t="n">
         <v>3</v>
       </c>
       <c r="Q96" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="R96" t="n">
         <v>2.44</v>
@@ -7012,7 +7012,7 @@
         </is>
       </c>
       <c r="K97" t="n">
-        <v>8.34</v>
+        <v>7.89</v>
       </c>
       <c r="L97" t="n">
         <v>3.06</v>
@@ -7024,13 +7024,13 @@
         <v>5.71</v>
       </c>
       <c r="O97" t="n">
-        <v>5.829499999999999</v>
+        <v>5.6945</v>
       </c>
       <c r="P97" t="n">
         <v>2</v>
       </c>
       <c r="Q97" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="R97" t="n">
         <v>2.603</v>
@@ -7080,7 +7080,7 @@
         </is>
       </c>
       <c r="K98" t="n">
-        <v>7.86</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="L98" t="n">
         <v>7.2</v>
@@ -7092,13 +7092,13 @@
         <v>10</v>
       </c>
       <c r="O98" t="n">
-        <v>8.378</v>
+        <v>8.431999999999999</v>
       </c>
       <c r="P98" t="n">
         <v>1</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.253</v>
+        <v>0.2334</v>
       </c>
       <c r="R98" t="n">
         <v>1.197</v>
@@ -7148,7 +7148,7 @@
         </is>
       </c>
       <c r="K99" t="n">
-        <v>9.32</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="L99" t="n">
         <v>7.2</v>
@@ -7160,13 +7160,13 @@
         <v>6.74</v>
       </c>
       <c r="O99" t="n">
-        <v>8.019</v>
+        <v>7.959000000000001</v>
       </c>
       <c r="P99" t="n">
         <v>2</v>
       </c>
       <c r="Q99" t="n">
-        <v>0.092</v>
+        <v>0.115</v>
       </c>
       <c r="R99" t="n">
         <v>1.197</v>
@@ -7216,7 +7216,7 @@
         </is>
       </c>
       <c r="K100" t="n">
-        <v>9.32</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="L100" t="n">
         <v>7.42</v>
@@ -7228,13 +7228,13 @@
         <v>3.6</v>
       </c>
       <c r="O100" t="n">
-        <v>7.351</v>
+        <v>7.291</v>
       </c>
       <c r="P100" t="n">
         <v>3</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.092</v>
+        <v>0.115</v>
       </c>
       <c r="R100" t="n">
         <v>1.122</v>
@@ -7488,7 +7488,7 @@
         </is>
       </c>
       <c r="K104" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L104" t="n">
         <v>5.97</v>
@@ -7500,7 +7500,7 @@
         <v>4.64</v>
       </c>
       <c r="O104" t="n">
-        <v>6.2775</v>
+        <v>6.280499999999999</v>
       </c>
       <c r="P104" t="n">
         <v>3</v>
@@ -7556,7 +7556,7 @@
         </is>
       </c>
       <c r="K105" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L105" t="n">
         <v>5.97</v>
@@ -7568,7 +7568,7 @@
         <v>3.63</v>
       </c>
       <c r="O105" t="n">
-        <v>6.358000000000001</v>
+        <v>6.361</v>
       </c>
       <c r="P105" t="n">
         <v>2</v>
@@ -7624,7 +7624,7 @@
         </is>
       </c>
       <c r="K106" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L106" t="n">
         <v>6.27</v>
@@ -7636,7 +7636,7 @@
         <v>3.48</v>
       </c>
       <c r="O106" t="n">
-        <v>6.5825</v>
+        <v>6.5855</v>
       </c>
       <c r="P106" t="n">
         <v>1</v>
@@ -7692,7 +7692,7 @@
         </is>
       </c>
       <c r="K107" t="n">
-        <v>10</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L107" t="n">
         <v>10</v>
@@ -7704,13 +7704,13 @@
         <v>9.25</v>
       </c>
       <c r="O107" t="n">
-        <v>9.797499999999999</v>
+        <v>9.788499999999999</v>
       </c>
       <c r="P107" t="n">
         <v>1</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.0158</v>
+        <v>0.0205</v>
       </c>
       <c r="R107" t="n">
         <v>0.229</v>
@@ -7760,7 +7760,7 @@
         </is>
       </c>
       <c r="K108" t="n">
-        <v>10</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L108" t="n">
         <v>10</v>
@@ -7772,13 +7772,13 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O108" t="n">
-        <v>9.5855</v>
+        <v>9.576499999999999</v>
       </c>
       <c r="P108" t="n">
         <v>2</v>
       </c>
       <c r="Q108" t="n">
-        <v>0.0158</v>
+        <v>0.0205</v>
       </c>
       <c r="R108" t="n">
         <v>0.229</v>
@@ -7828,7 +7828,7 @@
         </is>
       </c>
       <c r="K109" t="n">
-        <v>10</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="L109" t="n">
         <v>10</v>
@@ -7840,13 +7840,13 @@
         <v>6.69</v>
       </c>
       <c r="O109" t="n">
-        <v>9.069500000000001</v>
+        <v>9.060500000000001</v>
       </c>
       <c r="P109" t="n">
         <v>3</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.0158</v>
+        <v>0.0205</v>
       </c>
       <c r="R109" t="n">
         <v>0.229</v>
@@ -8100,7 +8100,7 @@
         </is>
       </c>
       <c r="K113" t="n">
-        <v>9.83</v>
+        <v>9.75</v>
       </c>
       <c r="L113" t="n">
         <v>9.34</v>
@@ -8112,13 +8112,13 @@
         <v>9.17</v>
       </c>
       <c r="O113" t="n">
-        <v>9.4915</v>
+        <v>9.467499999999999</v>
       </c>
       <c r="P113" t="n">
         <v>1</v>
       </c>
       <c r="Q113" t="n">
-        <v>0.036</v>
+        <v>0.045</v>
       </c>
       <c r="R113" t="n">
         <v>0.468</v>
@@ -8168,7 +8168,7 @@
         </is>
       </c>
       <c r="K114" t="n">
-        <v>9.83</v>
+        <v>9.75</v>
       </c>
       <c r="L114" t="n">
         <v>9.34</v>
@@ -8180,13 +8180,13 @@
         <v>8.289999999999999</v>
       </c>
       <c r="O114" t="n">
-        <v>9.251499999999998</v>
+        <v>9.227499999999999</v>
       </c>
       <c r="P114" t="n">
         <v>2</v>
       </c>
       <c r="Q114" t="n">
-        <v>0.036</v>
+        <v>0.045</v>
       </c>
       <c r="R114" t="n">
         <v>0.468</v>
@@ -8236,7 +8236,7 @@
         </is>
       </c>
       <c r="K115" t="n">
-        <v>9.26</v>
+        <v>9.33</v>
       </c>
       <c r="L115" t="n">
         <v>9.34</v>
@@ -8248,13 +8248,13 @@
         <v>5.61</v>
       </c>
       <c r="O115" t="n">
-        <v>8.272500000000001</v>
+        <v>8.2935</v>
       </c>
       <c r="P115" t="n">
         <v>3</v>
       </c>
       <c r="Q115" t="n">
-        <v>0.099</v>
+        <v>0.0914</v>
       </c>
       <c r="R115" t="n">
         <v>0.468</v>
@@ -8304,7 +8304,7 @@
         </is>
       </c>
       <c r="K116" t="n">
-        <v>9.890000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="L116" t="n">
         <v>9.550000000000001</v>
@@ -8316,7 +8316,7 @@
         <v>9.1</v>
       </c>
       <c r="O116" t="n">
-        <v>9.560499999999999</v>
+        <v>9.563499999999999</v>
       </c>
       <c r="P116" t="n">
         <v>1</v>
@@ -8372,7 +8372,7 @@
         </is>
       </c>
       <c r="K117" t="n">
-        <v>9.890000000000001</v>
+        <v>9.9</v>
       </c>
       <c r="L117" t="n">
         <v>9.550000000000001</v>
@@ -8384,7 +8384,7 @@
         <v>7.32</v>
       </c>
       <c r="O117" t="n">
-        <v>9.0435</v>
+        <v>9.0465</v>
       </c>
       <c r="P117" t="n">
         <v>2</v>
@@ -8440,7 +8440,7 @@
         </is>
       </c>
       <c r="K118" t="n">
-        <v>9.050000000000001</v>
+        <v>9.06</v>
       </c>
       <c r="L118" t="n">
         <v>9.550000000000001</v>
@@ -8452,7 +8452,7 @@
         <v>4.64</v>
       </c>
       <c r="O118" t="n">
-        <v>7.915500000000001</v>
+        <v>7.9185</v>
       </c>
       <c r="P118" t="n">
         <v>3</v>
@@ -8508,7 +8508,7 @@
         </is>
       </c>
       <c r="K119" t="n">
-        <v>8.33</v>
+        <v>7.8</v>
       </c>
       <c r="L119" t="n">
         <v>2.14</v>
@@ -8520,13 +8520,13 @@
         <v>9.15</v>
       </c>
       <c r="O119" t="n">
-        <v>6.512500000000001</v>
+        <v>6.3535</v>
       </c>
       <c r="P119" t="n">
         <v>1</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.2016</v>
+        <v>0.2604</v>
       </c>
       <c r="R119" t="n">
         <v>2.915</v>
@@ -8576,7 +8576,7 @@
         </is>
       </c>
       <c r="K120" t="n">
-        <v>8.33</v>
+        <v>7.8</v>
       </c>
       <c r="L120" t="n">
         <v>2.14</v>
@@ -8588,13 +8588,13 @@
         <v>8.23</v>
       </c>
       <c r="O120" t="n">
-        <v>6.2625</v>
+        <v>6.103499999999999</v>
       </c>
       <c r="P120" t="n">
         <v>2</v>
       </c>
       <c r="Q120" t="n">
-        <v>0.2016</v>
+        <v>0.2604</v>
       </c>
       <c r="R120" t="n">
         <v>2.915</v>
@@ -8712,7 +8712,7 @@
         </is>
       </c>
       <c r="K122" t="n">
-        <v>7.87</v>
+        <v>7.21</v>
       </c>
       <c r="L122" t="n">
         <v>0</v>
@@ -8724,13 +8724,13 @@
         <v>10</v>
       </c>
       <c r="O122" t="n">
-        <v>5.861</v>
+        <v>5.663</v>
       </c>
       <c r="P122" t="n">
         <v>1</v>
       </c>
       <c r="Q122" t="n">
-        <v>0.252</v>
+        <v>0.3255</v>
       </c>
       <c r="R122" t="n">
         <v>3.643</v>
@@ -8780,7 +8780,7 @@
         </is>
       </c>
       <c r="K123" t="n">
-        <v>7.87</v>
+        <v>7.21</v>
       </c>
       <c r="L123" t="n">
         <v>0</v>
@@ -8792,13 +8792,13 @@
         <v>6.66</v>
       </c>
       <c r="O123" t="n">
-        <v>4.922</v>
+        <v>4.723999999999999</v>
       </c>
       <c r="P123" t="n">
         <v>2</v>
       </c>
       <c r="Q123" t="n">
-        <v>0.252</v>
+        <v>0.3255</v>
       </c>
       <c r="R123" t="n">
         <v>3.643</v>
@@ -8848,7 +8848,7 @@
         </is>
       </c>
       <c r="K124" t="n">
-        <v>4.28</v>
+        <v>4.29</v>
       </c>
       <c r="L124" t="n">
         <v>0</v>
@@ -8860,7 +8860,7 @@
         <v>4.31</v>
       </c>
       <c r="O124" t="n">
-        <v>3.1145</v>
+        <v>3.1175</v>
       </c>
       <c r="P124" t="n">
         <v>3</v>
@@ -8916,7 +8916,7 @@
         </is>
       </c>
       <c r="K125" t="n">
-        <v>6.98</v>
+        <v>7.94</v>
       </c>
       <c r="L125" t="n">
         <v>0</v>
@@ -8928,13 +8928,13 @@
         <v>10</v>
       </c>
       <c r="O125" t="n">
-        <v>5.593999999999999</v>
+        <v>5.882</v>
       </c>
       <c r="P125" t="n">
         <v>1</v>
       </c>
       <c r="Q125" t="n">
-        <v>0.35</v>
+        <v>0.245</v>
       </c>
       <c r="R125" t="n">
         <v>3.643</v>
@@ -8984,7 +8984,7 @@
         </is>
       </c>
       <c r="K126" t="n">
-        <v>6.98</v>
+        <v>7.94</v>
       </c>
       <c r="L126" t="n">
         <v>0</v>
@@ -8996,13 +8996,13 @@
         <v>7.82</v>
       </c>
       <c r="O126" t="n">
-        <v>4.987</v>
+        <v>5.275</v>
       </c>
       <c r="P126" t="n">
         <v>2</v>
       </c>
       <c r="Q126" t="n">
-        <v>0.35</v>
+        <v>0.245</v>
       </c>
       <c r="R126" t="n">
         <v>3.643</v>
@@ -9052,7 +9052,7 @@
         </is>
       </c>
       <c r="K127" t="n">
-        <v>5.71</v>
+        <v>5.08</v>
       </c>
       <c r="L127" t="n">
         <v>0</v>
@@ -9064,13 +9064,13 @@
         <v>6.21</v>
       </c>
       <c r="O127" t="n">
-        <v>4.1305</v>
+        <v>3.9415</v>
       </c>
       <c r="P127" t="n">
         <v>3</v>
       </c>
       <c r="Q127" t="n">
-        <v>0.49</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="R127" t="n">
         <v>3.643</v>
@@ -9120,7 +9120,7 @@
         </is>
       </c>
       <c r="K128" t="n">
-        <v>9.289999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L128" t="n">
         <v>6.89</v>
@@ -9132,7 +9132,7 @@
         <v>10</v>
       </c>
       <c r="O128" t="n">
-        <v>8.698499999999999</v>
+        <v>8.701499999999999</v>
       </c>
       <c r="P128" t="n">
         <v>1</v>
@@ -9256,7 +9256,7 @@
         </is>
       </c>
       <c r="K130" t="n">
-        <v>9.289999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L130" t="n">
         <v>7.13</v>
@@ -9268,7 +9268,7 @@
         <v>1.71</v>
       </c>
       <c r="O130" t="n">
-        <v>6.494999999999999</v>
+        <v>6.498</v>
       </c>
       <c r="P130" t="n">
         <v>3</v>
@@ -9324,7 +9324,7 @@
         </is>
       </c>
       <c r="K131" t="n">
-        <v>9.84</v>
+        <v>9.94</v>
       </c>
       <c r="L131" t="n">
         <v>9.65</v>
@@ -9336,13 +9336,13 @@
         <v>10</v>
       </c>
       <c r="O131" t="n">
-        <v>9.829499999999999</v>
+        <v>9.859500000000001</v>
       </c>
       <c r="P131" t="n">
         <v>1</v>
       </c>
       <c r="Q131" t="n">
-        <v>0.035</v>
+        <v>0.0245</v>
       </c>
       <c r="R131" t="n">
         <v>0.364</v>
@@ -9392,7 +9392,7 @@
         </is>
       </c>
       <c r="K132" t="n">
-        <v>9.710000000000001</v>
+        <v>9.65</v>
       </c>
       <c r="L132" t="n">
         <v>9.65</v>
@@ -9404,13 +9404,13 @@
         <v>5.61</v>
       </c>
       <c r="O132" t="n">
-        <v>8.516</v>
+        <v>8.498000000000001</v>
       </c>
       <c r="P132" t="n">
         <v>2</v>
       </c>
       <c r="Q132" t="n">
-        <v>0.049</v>
+        <v>0.056</v>
       </c>
       <c r="R132" t="n">
         <v>0.364</v>
@@ -9460,7 +9460,7 @@
         </is>
       </c>
       <c r="K133" t="n">
-        <v>9.84</v>
+        <v>9.94</v>
       </c>
       <c r="L133" t="n">
         <v>9.710000000000001</v>
@@ -9472,13 +9472,13 @@
         <v>1.51</v>
       </c>
       <c r="O133" t="n">
-        <v>7.343</v>
+        <v>7.372999999999999</v>
       </c>
       <c r="P133" t="n">
         <v>3</v>
       </c>
       <c r="Q133" t="n">
-        <v>0.035</v>
+        <v>0.0245</v>
       </c>
       <c r="R133" t="n">
         <v>0.342</v>
@@ -9528,7 +9528,7 @@
         </is>
       </c>
       <c r="K134" t="n">
-        <v>7.89</v>
+        <v>8.57</v>
       </c>
       <c r="L134" t="n">
         <v>3.06</v>
@@ -9540,13 +9540,13 @@
         <v>10</v>
       </c>
       <c r="O134" t="n">
-        <v>6.938</v>
+        <v>7.142</v>
       </c>
       <c r="P134" t="n">
         <v>1</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.25</v>
+        <v>0.175</v>
       </c>
       <c r="R134" t="n">
         <v>2.603</v>
@@ -9596,7 +9596,7 @@
         </is>
       </c>
       <c r="K135" t="n">
-        <v>7.89</v>
+        <v>8.57</v>
       </c>
       <c r="L135" t="n">
         <v>3.06</v>
@@ -9608,13 +9608,13 @@
         <v>3.42</v>
       </c>
       <c r="O135" t="n">
-        <v>4.976999999999999</v>
+        <v>5.181</v>
       </c>
       <c r="P135" t="n">
         <v>2</v>
       </c>
       <c r="Q135" t="n">
-        <v>0.25</v>
+        <v>0.175</v>
       </c>
       <c r="R135" t="n">
         <v>2.603</v>
@@ -9664,7 +9664,7 @@
         </is>
       </c>
       <c r="K136" t="n">
-        <v>7.89</v>
+        <v>8.57</v>
       </c>
       <c r="L136" t="n">
         <v>3.54</v>
@@ -9676,13 +9676,13 @@
         <v>1.79</v>
       </c>
       <c r="O136" t="n">
-        <v>4.7305</v>
+        <v>4.934500000000001</v>
       </c>
       <c r="P136" t="n">
         <v>3</v>
       </c>
       <c r="Q136" t="n">
-        <v>0.25</v>
+        <v>0.175</v>
       </c>
       <c r="R136" t="n">
         <v>2.44</v>
@@ -9800,7 +9800,7 @@
         </is>
       </c>
       <c r="K138" t="n">
-        <v>6.96</v>
+        <v>6.97</v>
       </c>
       <c r="L138" t="n">
         <v>7.35</v>
@@ -9812,7 +9812,7 @@
         <v>6.69</v>
       </c>
       <c r="O138" t="n">
-        <v>7.23</v>
+        <v>7.232999999999999</v>
       </c>
       <c r="P138" t="n">
         <v>3</v>
@@ -9936,7 +9936,7 @@
         </is>
       </c>
       <c r="K140" t="n">
-        <v>9.75</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="L140" t="n">
         <v>9.34</v>
@@ -9948,13 +9948,13 @@
         <v>10</v>
       </c>
       <c r="O140" t="n">
-        <v>9.693999999999999</v>
+        <v>9.73</v>
       </c>
       <c r="P140" t="n">
         <v>1</v>
       </c>
       <c r="Q140" t="n">
-        <v>0.045</v>
+        <v>0.0315</v>
       </c>
       <c r="R140" t="n">
         <v>0.468</v>
@@ -10004,7 +10004,7 @@
         </is>
       </c>
       <c r="K141" t="n">
-        <v>9.75</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="L141" t="n">
         <v>9.34</v>
@@ -10016,13 +10016,13 @@
         <v>2.95</v>
       </c>
       <c r="O141" t="n">
-        <v>7.578499999999999</v>
+        <v>7.6145</v>
       </c>
       <c r="P141" t="n">
         <v>2</v>
       </c>
       <c r="Q141" t="n">
-        <v>0.045</v>
+        <v>0.0315</v>
       </c>
       <c r="R141" t="n">
         <v>0.468</v>
@@ -10072,7 +10072,7 @@
         </is>
       </c>
       <c r="K142" t="n">
-        <v>9.75</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="L142" t="n">
         <v>9.43</v>
@@ -10084,13 +10084,13 @@
         <v>1.51</v>
       </c>
       <c r="O142" t="n">
-        <v>7.023999999999999</v>
+        <v>7.06</v>
       </c>
       <c r="P142" t="n">
         <v>3</v>
       </c>
       <c r="Q142" t="n">
-        <v>0.045</v>
+        <v>0.0315</v>
       </c>
       <c r="R142" t="n">
         <v>0.439</v>
@@ -10548,7 +10548,7 @@
         </is>
       </c>
       <c r="K149" t="n">
-        <v>6.66</v>
+        <v>6.67</v>
       </c>
       <c r="L149" t="n">
         <v>2.14</v>
@@ -10560,7 +10560,7 @@
         <v>10</v>
       </c>
       <c r="O149" t="n">
-        <v>6.247</v>
+        <v>6.25</v>
       </c>
       <c r="P149" t="n">
         <v>1</v>
@@ -10616,7 +10616,7 @@
         </is>
       </c>
       <c r="K150" t="n">
-        <v>6.66</v>
+        <v>6.67</v>
       </c>
       <c r="L150" t="n">
         <v>2.14</v>
@@ -10628,7 +10628,7 @@
         <v>6.04</v>
       </c>
       <c r="O150" t="n">
-        <v>5.111</v>
+        <v>5.114</v>
       </c>
       <c r="P150" t="n">
         <v>2</v>
@@ -10684,7 +10684,7 @@
         </is>
       </c>
       <c r="K151" t="n">
-        <v>6.66</v>
+        <v>6.67</v>
       </c>
       <c r="L151" t="n">
         <v>2.68</v>
@@ -10696,7 +10696,7 @@
         <v>2.13</v>
       </c>
       <c r="O151" t="n">
-        <v>3.7255</v>
+        <v>3.7285</v>
       </c>
       <c r="P151" t="n">
         <v>3</v>
@@ -11160,7 +11160,7 @@
         </is>
       </c>
       <c r="K158" t="n">
-        <v>9.9</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="L158" t="n">
         <v>10</v>
@@ -11172,13 +11172,13 @@
         <v>10</v>
       </c>
       <c r="O158" t="n">
-        <v>9.970000000000001</v>
+        <v>9.961</v>
       </c>
       <c r="P158" t="n">
         <v>1</v>
       </c>
       <c r="Q158" t="n">
-        <v>0.028</v>
+        <v>0.032</v>
       </c>
       <c r="R158" t="n">
         <v>0.208</v>
@@ -11228,7 +11228,7 @@
         </is>
       </c>
       <c r="K159" t="n">
-        <v>9.970000000000001</v>
+        <v>10</v>
       </c>
       <c r="L159" t="n">
         <v>10</v>
@@ -11240,13 +11240,13 @@
         <v>5.71</v>
       </c>
       <c r="O159" t="n">
-        <v>8.7475</v>
+        <v>8.756500000000001</v>
       </c>
       <c r="P159" t="n">
         <v>2</v>
       </c>
       <c r="Q159" t="n">
-        <v>0.02</v>
+        <v>0.014</v>
       </c>
       <c r="R159" t="n">
         <v>0.208</v>
@@ -11296,7 +11296,7 @@
         </is>
       </c>
       <c r="K160" t="n">
-        <v>9.970000000000001</v>
+        <v>10</v>
       </c>
       <c r="L160" t="n">
         <v>10</v>
@@ -11308,13 +11308,13 @@
         <v>2.86</v>
       </c>
       <c r="O160" t="n">
-        <v>7.638</v>
+        <v>7.647</v>
       </c>
       <c r="P160" t="n">
         <v>3</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.02</v>
+        <v>0.014</v>
       </c>
       <c r="R160" t="n">
         <v>0.195</v>
@@ -11364,7 +11364,7 @@
         </is>
       </c>
       <c r="K161" t="n">
-        <v>9.859999999999999</v>
+        <v>9.82</v>
       </c>
       <c r="L161" t="n">
         <v>10</v>
@@ -11376,13 +11376,13 @@
         <v>10</v>
       </c>
       <c r="O161" t="n">
-        <v>9.958</v>
+        <v>9.946</v>
       </c>
       <c r="P161" t="n">
         <v>1</v>
       </c>
       <c r="Q161" t="n">
-        <v>0.0322</v>
+        <v>0.0368</v>
       </c>
       <c r="R161" t="n">
         <v>0.239</v>
@@ -11432,7 +11432,7 @@
         </is>
       </c>
       <c r="K162" t="n">
-        <v>9.949999999999999</v>
+        <v>10</v>
       </c>
       <c r="L162" t="n">
         <v>10</v>
@@ -11444,13 +11444,13 @@
         <v>4.64</v>
       </c>
       <c r="O162" t="n">
-        <v>8.365</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="P162" t="n">
         <v>3</v>
       </c>
       <c r="Q162" t="n">
-        <v>0.023</v>
+        <v>0.0161</v>
       </c>
       <c r="R162" t="n">
         <v>0.239</v>
@@ -11500,7 +11500,7 @@
         </is>
       </c>
       <c r="K163" t="n">
-        <v>9.949999999999999</v>
+        <v>10</v>
       </c>
       <c r="L163" t="n">
         <v>10</v>
@@ -11512,13 +11512,13 @@
         <v>5.19</v>
       </c>
       <c r="O163" t="n">
-        <v>8.465499999999999</v>
+        <v>8.480499999999999</v>
       </c>
       <c r="P163" t="n">
         <v>2</v>
       </c>
       <c r="Q163" t="n">
-        <v>0.023</v>
+        <v>0.0161</v>
       </c>
       <c r="R163" t="n">
         <v>0.239</v>
@@ -11772,7 +11772,7 @@
         </is>
       </c>
       <c r="K167" t="n">
-        <v>6.98</v>
+        <v>7.94</v>
       </c>
       <c r="L167" t="n">
         <v>0</v>
@@ -11784,13 +11784,13 @@
         <v>10</v>
       </c>
       <c r="O167" t="n">
-        <v>5.593999999999999</v>
+        <v>5.882</v>
       </c>
       <c r="P167" t="n">
         <v>1</v>
       </c>
       <c r="Q167" t="n">
-        <v>0.35</v>
+        <v>0.245</v>
       </c>
       <c r="R167" t="n">
         <v>3.643</v>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
       <c r="K168" t="n">
-        <v>6.98</v>
+        <v>7.94</v>
       </c>
       <c r="L168" t="n">
         <v>0</v>
@@ -11852,13 +11852,13 @@
         <v>3.42</v>
       </c>
       <c r="O168" t="n">
-        <v>3.633</v>
+        <v>3.921</v>
       </c>
       <c r="P168" t="n">
         <v>3</v>
       </c>
       <c r="Q168" t="n">
-        <v>0.35</v>
+        <v>0.245</v>
       </c>
       <c r="R168" t="n">
         <v>3.643</v>
@@ -11908,7 +11908,7 @@
         </is>
       </c>
       <c r="K169" t="n">
-        <v>6.98</v>
+        <v>7.94</v>
       </c>
       <c r="L169" t="n">
         <v>0.67</v>
@@ -11920,13 +11920,13 @@
         <v>3.88</v>
       </c>
       <c r="O169" t="n">
-        <v>3.9225</v>
+        <v>4.210500000000001</v>
       </c>
       <c r="P169" t="n">
         <v>2</v>
       </c>
       <c r="Q169" t="n">
-        <v>0.35</v>
+        <v>0.245</v>
       </c>
       <c r="R169" t="n">
         <v>3.416</v>
@@ -12180,7 +12180,7 @@
         </is>
       </c>
       <c r="K173" t="n">
-        <v>9.81</v>
+        <v>9.92</v>
       </c>
       <c r="L173" t="n">
         <v>9.630000000000001</v>
@@ -12192,13 +12192,13 @@
         <v>9.25</v>
       </c>
       <c r="O173" t="n">
-        <v>9.266999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="P173" t="n">
         <v>1</v>
       </c>
       <c r="Q173" t="n">
-        <v>0.038</v>
+        <v>0.0266</v>
       </c>
       <c r="R173" t="n">
         <v>0.371</v>
@@ -12248,7 +12248,7 @@
         </is>
       </c>
       <c r="K174" t="n">
-        <v>9.81</v>
+        <v>9.92</v>
       </c>
       <c r="L174" t="n">
         <v>9.550000000000001</v>
@@ -12260,13 +12260,13 @@
         <v>3.87</v>
       </c>
       <c r="O174" t="n">
-        <v>7.972</v>
+        <v>8.005000000000001</v>
       </c>
       <c r="P174" t="n">
         <v>2</v>
       </c>
       <c r="Q174" t="n">
-        <v>0.038</v>
+        <v>0.0266</v>
       </c>
       <c r="R174" t="n">
         <v>0.396</v>
@@ -12316,7 +12316,7 @@
         </is>
       </c>
       <c r="K175" t="n">
-        <v>9.67</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="L175" t="n">
         <v>9.550000000000001</v>
@@ -12328,13 +12328,13 @@
         <v>3.87</v>
       </c>
       <c r="O175" t="n">
-        <v>7.93</v>
+        <v>7.912</v>
       </c>
       <c r="P175" t="n">
         <v>3</v>
       </c>
       <c r="Q175" t="n">
-        <v>0.0532</v>
+        <v>0.0608</v>
       </c>
       <c r="R175" t="n">
         <v>0.396</v>
@@ -12384,7 +12384,7 @@
         </is>
       </c>
       <c r="K176" t="n">
-        <v>8.43</v>
+        <v>8.44</v>
       </c>
       <c r="L176" t="n">
         <v>3.06</v>
@@ -12396,7 +12396,7 @@
         <v>9.25</v>
       </c>
       <c r="O176" t="n">
-        <v>6.5535</v>
+        <v>6.5565</v>
       </c>
       <c r="P176" t="n">
         <v>1</v>
@@ -12452,7 +12452,7 @@
         </is>
       </c>
       <c r="K177" t="n">
-        <v>8.43</v>
+        <v>8.44</v>
       </c>
       <c r="L177" t="n">
         <v>3.06</v>
@@ -12464,7 +12464,7 @@
         <v>2.95</v>
       </c>
       <c r="O177" t="n">
-        <v>4.9845</v>
+        <v>4.9875</v>
       </c>
       <c r="P177" t="n">
         <v>2</v>
@@ -12588,7 +12588,7 @@
         </is>
       </c>
       <c r="K179" t="n">
-        <v>9.9</v>
+        <v>9.84</v>
       </c>
       <c r="L179" t="n">
         <v>9.710000000000001</v>
@@ -12600,13 +12600,13 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O179" t="n">
-        <v>9.202</v>
+        <v>9.183999999999999</v>
       </c>
       <c r="P179" t="n">
         <v>1</v>
       </c>
       <c r="Q179" t="n">
-        <v>0.028</v>
+        <v>0.035</v>
       </c>
       <c r="R179" t="n">
         <v>0.342</v>
@@ -12656,7 +12656,7 @@
         </is>
       </c>
       <c r="K180" t="n">
-        <v>9.9</v>
+        <v>9.84</v>
       </c>
       <c r="L180" t="n">
         <v>9.65</v>
@@ -12668,13 +12668,13 @@
         <v>4.36</v>
       </c>
       <c r="O180" t="n">
-        <v>8.185500000000001</v>
+        <v>8.1675</v>
       </c>
       <c r="P180" t="n">
         <v>3</v>
       </c>
       <c r="Q180" t="n">
-        <v>0.028</v>
+        <v>0.035</v>
       </c>
       <c r="R180" t="n">
         <v>0.364</v>
@@ -12724,7 +12724,7 @@
         </is>
       </c>
       <c r="K181" t="n">
-        <v>9.460000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="L181" t="n">
         <v>9.65</v>
@@ -12736,13 +12736,13 @@
         <v>4.78</v>
       </c>
       <c r="O181" t="n">
-        <v>8.1905</v>
+        <v>8.205499999999999</v>
       </c>
       <c r="P181" t="n">
         <v>2</v>
       </c>
       <c r="Q181" t="n">
-        <v>0.077</v>
+        <v>0.0711</v>
       </c>
       <c r="R181" t="n">
         <v>0.364</v>
@@ -12792,7 +12792,7 @@
         </is>
       </c>
       <c r="K182" t="n">
-        <v>8.199999999999999</v>
+        <v>7.63</v>
       </c>
       <c r="L182" t="n">
         <v>2.11</v>
@@ -12804,13 +12804,13 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O182" t="n">
-        <v>6.031999999999999</v>
+        <v>5.861</v>
       </c>
       <c r="P182" t="n">
         <v>1</v>
       </c>
       <c r="Q182" t="n">
-        <v>0.216</v>
+        <v>0.279</v>
       </c>
       <c r="R182" t="n">
         <v>2.928</v>
@@ -12860,7 +12860,7 @@
         </is>
       </c>
       <c r="K183" t="n">
-        <v>8.199999999999999</v>
+        <v>7.63</v>
       </c>
       <c r="L183" t="n">
         <v>1.53</v>
@@ -12872,13 +12872,13 @@
         <v>5.19</v>
       </c>
       <c r="O183" t="n">
-        <v>5.104</v>
+        <v>4.933</v>
       </c>
       <c r="P183" t="n">
         <v>2</v>
       </c>
       <c r="Q183" t="n">
-        <v>0.216</v>
+        <v>0.279</v>
       </c>
       <c r="R183" t="n">
         <v>3.123</v>
@@ -12996,7 +12996,7 @@
         </is>
       </c>
       <c r="K185" t="n">
-        <v>9.880000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L185" t="n">
         <v>9.43</v>
@@ -13008,13 +13008,13 @@
         <v>9.25</v>
       </c>
       <c r="O185" t="n">
-        <v>9.311999999999999</v>
+        <v>9.287999999999998</v>
       </c>
       <c r="P185" t="n">
         <v>1</v>
       </c>
       <c r="Q185" t="n">
-        <v>0.0302</v>
+        <v>0.0396</v>
       </c>
       <c r="R185" t="n">
         <v>0.439</v>
@@ -13064,7 +13064,7 @@
         </is>
       </c>
       <c r="K186" t="n">
-        <v>9.880000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L186" t="n">
         <v>9.34</v>
@@ -13076,13 +13076,13 @@
         <v>3.87</v>
       </c>
       <c r="O186" t="n">
-        <v>7.919499999999999</v>
+        <v>7.895499999999999</v>
       </c>
       <c r="P186" t="n">
         <v>3</v>
       </c>
       <c r="Q186" t="n">
-        <v>0.0302</v>
+        <v>0.0396</v>
       </c>
       <c r="R186" t="n">
         <v>0.468</v>
@@ -13132,7 +13132,7 @@
         </is>
       </c>
       <c r="K187" t="n">
-        <v>9.48</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L187" t="n">
         <v>9.34</v>
@@ -13144,13 +13144,13 @@
         <v>4.64</v>
       </c>
       <c r="O187" t="n">
-        <v>7.992999999999999</v>
+        <v>7.986999999999999</v>
       </c>
       <c r="P187" t="n">
         <v>2</v>
       </c>
       <c r="Q187" t="n">
-        <v>0.0743</v>
+        <v>0.0774</v>
       </c>
       <c r="R187" t="n">
         <v>0.468</v>
@@ -13200,7 +13200,7 @@
         </is>
       </c>
       <c r="K188" t="n">
-        <v>9.289999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L188" t="n">
         <v>6.89</v>
@@ -13212,7 +13212,7 @@
         <v>10</v>
       </c>
       <c r="O188" t="n">
-        <v>8.698499999999999</v>
+        <v>8.701499999999999</v>
       </c>
       <c r="P188" t="n">
         <v>1</v>
@@ -13268,7 +13268,7 @@
         </is>
       </c>
       <c r="K189" t="n">
-        <v>9.289999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L189" t="n">
         <v>6.89</v>
@@ -13280,7 +13280,7 @@
         <v>6.69</v>
       </c>
       <c r="O189" t="n">
-        <v>7.767999999999999</v>
+        <v>7.770999999999999</v>
       </c>
       <c r="P189" t="n">
         <v>2</v>
@@ -13336,7 +13336,7 @@
         </is>
       </c>
       <c r="K190" t="n">
-        <v>9.289999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L190" t="n">
         <v>6.89</v>
@@ -13348,7 +13348,7 @@
         <v>4.64</v>
       </c>
       <c r="O190" t="n">
-        <v>6.826499999999999</v>
+        <v>6.829499999999999</v>
       </c>
       <c r="P190" t="n">
         <v>3</v>
@@ -13404,7 +13404,7 @@
         </is>
       </c>
       <c r="K191" t="n">
-        <v>6.98</v>
+        <v>6.53</v>
       </c>
       <c r="L191" t="n">
         <v>3.06</v>
@@ -13416,13 +13416,13 @@
         <v>10</v>
       </c>
       <c r="O191" t="n">
-        <v>6.665</v>
+        <v>6.53</v>
       </c>
       <c r="P191" t="n">
         <v>1</v>
       </c>
       <c r="Q191" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="R191" t="n">
         <v>2.603</v>
@@ -13472,7 +13472,7 @@
         </is>
       </c>
       <c r="K192" t="n">
-        <v>6.98</v>
+        <v>6.53</v>
       </c>
       <c r="L192" t="n">
         <v>3.06</v>
@@ -13484,13 +13484,13 @@
         <v>8.029999999999999</v>
       </c>
       <c r="O192" t="n">
-        <v>6.115500000000001</v>
+        <v>5.980500000000001</v>
       </c>
       <c r="P192" t="n">
         <v>2</v>
       </c>
       <c r="Q192" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="R192" t="n">
         <v>2.603</v>
@@ -13540,7 +13540,7 @@
         </is>
       </c>
       <c r="K193" t="n">
-        <v>7.89</v>
+        <v>8.57</v>
       </c>
       <c r="L193" t="n">
         <v>3.06</v>
@@ -13552,13 +13552,13 @@
         <v>4.64</v>
       </c>
       <c r="O193" t="n">
-        <v>5.356</v>
+        <v>5.56</v>
       </c>
       <c r="P193" t="n">
         <v>3</v>
       </c>
       <c r="Q193" t="n">
-        <v>0.25</v>
+        <v>0.175</v>
       </c>
       <c r="R193" t="n">
         <v>2.603</v>
@@ -13608,7 +13608,7 @@
         </is>
       </c>
       <c r="K194" t="n">
-        <v>9.16</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L194" t="n">
         <v>7.35</v>
@@ -13620,13 +13620,13 @@
         <v>10</v>
       </c>
       <c r="O194" t="n">
-        <v>8.820499999999999</v>
+        <v>8.910499999999999</v>
       </c>
       <c r="P194" t="n">
         <v>1</v>
       </c>
       <c r="Q194" t="n">
-        <v>0.11</v>
+        <v>0.077</v>
       </c>
       <c r="R194" t="n">
         <v>1.145</v>
@@ -13676,7 +13676,7 @@
         </is>
       </c>
       <c r="K195" t="n">
-        <v>8.76</v>
+        <v>8.56</v>
       </c>
       <c r="L195" t="n">
         <v>7.35</v>
@@ -13688,13 +13688,13 @@
         <v>5.81</v>
       </c>
       <c r="O195" t="n">
-        <v>7.49</v>
+        <v>7.43</v>
       </c>
       <c r="P195" t="n">
         <v>2</v>
       </c>
       <c r="Q195" t="n">
-        <v>0.154</v>
+        <v>0.176</v>
       </c>
       <c r="R195" t="n">
         <v>1.145</v>
@@ -13744,7 +13744,7 @@
         </is>
       </c>
       <c r="K196" t="n">
-        <v>9.16</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L196" t="n">
         <v>7.35</v>
@@ -13756,13 +13756,13 @@
         <v>4.64</v>
       </c>
       <c r="O196" t="n">
-        <v>6.972499999999999</v>
+        <v>7.0625</v>
       </c>
       <c r="P196" t="n">
         <v>3</v>
       </c>
       <c r="Q196" t="n">
-        <v>0.11</v>
+        <v>0.077</v>
       </c>
       <c r="R196" t="n">
         <v>1.145</v>
@@ -13812,7 +13812,7 @@
         </is>
       </c>
       <c r="K197" t="n">
-        <v>9.81</v>
+        <v>9.92</v>
       </c>
       <c r="L197" t="n">
         <v>9.630000000000001</v>
@@ -13824,13 +13824,13 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O197" t="n">
-        <v>9.147</v>
+        <v>9.18</v>
       </c>
       <c r="P197" t="n">
         <v>1</v>
       </c>
       <c r="Q197" t="n">
-        <v>0.038</v>
+        <v>0.0266</v>
       </c>
       <c r="R197" t="n">
         <v>0.371</v>
@@ -13880,7 +13880,7 @@
         </is>
       </c>
       <c r="K198" t="n">
-        <v>9.81</v>
+        <v>9.92</v>
       </c>
       <c r="L198" t="n">
         <v>9.550000000000001</v>
@@ -13892,13 +13892,13 @@
         <v>4.64</v>
       </c>
       <c r="O198" t="n">
-        <v>8.027500000000002</v>
+        <v>8.060500000000001</v>
       </c>
       <c r="P198" t="n">
         <v>2</v>
       </c>
       <c r="Q198" t="n">
-        <v>0.038</v>
+        <v>0.0266</v>
       </c>
       <c r="R198" t="n">
         <v>0.396</v>
@@ -13948,7 +13948,7 @@
         </is>
       </c>
       <c r="K199" t="n">
-        <v>9.67</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="L199" t="n">
         <v>9.550000000000001</v>
@@ -13960,13 +13960,13 @@
         <v>2.03</v>
       </c>
       <c r="O199" t="n">
-        <v>7.336</v>
+        <v>7.318000000000001</v>
       </c>
       <c r="P199" t="n">
         <v>3</v>
       </c>
       <c r="Q199" t="n">
-        <v>0.0532</v>
+        <v>0.0608</v>
       </c>
       <c r="R199" t="n">
         <v>0.396</v>
@@ -14016,7 +14016,7 @@
         </is>
       </c>
       <c r="K200" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L200" t="n">
         <v>2.68</v>
@@ -14028,7 +14028,7 @@
         <v>8.449999999999999</v>
       </c>
       <c r="O200" t="n">
-        <v>6.2375</v>
+        <v>6.2405</v>
       </c>
       <c r="P200" t="n">
         <v>1</v>
@@ -14084,7 +14084,7 @@
         </is>
       </c>
       <c r="K201" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L201" t="n">
         <v>2.14</v>
@@ -14096,7 +14096,7 @@
         <v>4.08</v>
       </c>
       <c r="O201" t="n">
-        <v>4.953</v>
+        <v>4.956</v>
       </c>
       <c r="P201" t="n">
         <v>2</v>
@@ -14220,7 +14220,7 @@
         </is>
       </c>
       <c r="K203" t="n">
-        <v>8.34</v>
+        <v>7.89</v>
       </c>
       <c r="L203" t="n">
         <v>3.06</v>
@@ -14232,13 +14232,13 @@
         <v>10</v>
       </c>
       <c r="O203" t="n">
-        <v>7.073</v>
+        <v>6.938</v>
       </c>
       <c r="P203" t="n">
         <v>1</v>
       </c>
       <c r="Q203" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="R203" t="n">
         <v>2.603</v>
@@ -14288,7 +14288,7 @@
         </is>
       </c>
       <c r="K204" t="n">
-        <v>5.17</v>
+        <v>5.56</v>
       </c>
       <c r="L204" t="n">
         <v>3.06</v>
@@ -14300,13 +14300,13 @@
         <v>6.66</v>
       </c>
       <c r="O204" t="n">
-        <v>5.183</v>
+        <v>5.3</v>
       </c>
       <c r="P204" t="n">
         <v>2</v>
       </c>
       <c r="Q204" t="n">
-        <v>0.55</v>
+        <v>0.5075</v>
       </c>
       <c r="R204" t="n">
         <v>2.603</v>
@@ -14356,7 +14356,7 @@
         </is>
       </c>
       <c r="K205" t="n">
-        <v>8.34</v>
+        <v>7.89</v>
       </c>
       <c r="L205" t="n">
         <v>3.54</v>
@@ -14368,13 +14368,13 @@
         <v>1.51</v>
       </c>
       <c r="O205" t="n">
-        <v>4.539499999999999</v>
+        <v>4.4045</v>
       </c>
       <c r="P205" t="n">
         <v>3</v>
       </c>
       <c r="Q205" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="R205" t="n">
         <v>2.44</v>
@@ -14424,7 +14424,7 @@
         </is>
       </c>
       <c r="K206" t="n">
-        <v>9.92</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="L206" t="n">
         <v>9.74</v>
@@ -14436,13 +14436,13 @@
         <v>10</v>
       </c>
       <c r="O206" t="n">
-        <v>9.885</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="P206" t="n">
         <v>1</v>
       </c>
       <c r="Q206" t="n">
-        <v>0.0256</v>
+        <v>0.032</v>
       </c>
       <c r="R206" t="n">
         <v>0.333</v>
@@ -14492,7 +14492,7 @@
         </is>
       </c>
       <c r="K207" t="n">
-        <v>9.52</v>
+        <v>9.57</v>
       </c>
       <c r="L207" t="n">
         <v>9.74</v>
@@ -14504,13 +14504,13 @@
         <v>6.21</v>
       </c>
       <c r="O207" t="n">
-        <v>8.682499999999999</v>
+        <v>8.6975</v>
       </c>
       <c r="P207" t="n">
         <v>2</v>
       </c>
       <c r="Q207" t="n">
-        <v>0.0704</v>
+        <v>0.065</v>
       </c>
       <c r="R207" t="n">
         <v>0.333</v>
@@ -14560,7 +14560,7 @@
         </is>
       </c>
       <c r="K208" t="n">
-        <v>9.92</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="L208" t="n">
         <v>9.74</v>
@@ -14572,13 +14572,13 @@
         <v>2.2</v>
       </c>
       <c r="O208" t="n">
-        <v>7.021</v>
+        <v>7.005999999999999</v>
       </c>
       <c r="P208" t="n">
         <v>3</v>
       </c>
       <c r="Q208" t="n">
-        <v>0.0256</v>
+        <v>0.032</v>
       </c>
       <c r="R208" t="n">
         <v>0.333</v>
@@ -14628,7 +14628,7 @@
         </is>
       </c>
       <c r="K209" t="n">
-        <v>8.779999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="L209" t="n">
         <v>7.35</v>
@@ -14640,7 +14640,7 @@
         <v>10</v>
       </c>
       <c r="O209" t="n">
-        <v>8.7065</v>
+        <v>8.709499999999998</v>
       </c>
       <c r="P209" t="n">
         <v>1</v>
@@ -14696,7 +14696,7 @@
         </is>
       </c>
       <c r="K210" t="n">
-        <v>8.779999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="L210" t="n">
         <v>7.35</v>
@@ -14708,7 +14708,7 @@
         <v>4.64</v>
       </c>
       <c r="O210" t="n">
-        <v>6.7185</v>
+        <v>6.721499999999999</v>
       </c>
       <c r="P210" t="n">
         <v>3</v>
@@ -14764,7 +14764,7 @@
         </is>
       </c>
       <c r="K211" t="n">
-        <v>8.779999999999999</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="L211" t="n">
         <v>7.56</v>
@@ -14776,7 +14776,7 @@
         <v>6.57</v>
       </c>
       <c r="O211" t="n">
-        <v>7.929499999999999</v>
+        <v>7.932499999999999</v>
       </c>
       <c r="P211" t="n">
         <v>2</v>
@@ -15240,7 +15240,7 @@
         </is>
       </c>
       <c r="K218" t="n">
-        <v>9.880000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L218" t="n">
         <v>9.51</v>
@@ -15252,13 +15252,13 @@
         <v>9.25</v>
       </c>
       <c r="O218" t="n">
-        <v>9.245999999999999</v>
+        <v>9.222</v>
       </c>
       <c r="P218" t="n">
         <v>1</v>
       </c>
       <c r="Q218" t="n">
-        <v>0.0302</v>
+        <v>0.0391</v>
       </c>
       <c r="R218" t="n">
         <v>0.41</v>
@@ -15308,7 +15308,7 @@
         </is>
       </c>
       <c r="K219" t="n">
-        <v>9.880000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L219" t="n">
         <v>9.43</v>
@@ -15320,13 +15320,13 @@
         <v>2.95</v>
       </c>
       <c r="O219" t="n">
-        <v>7.649</v>
+        <v>7.624999999999999</v>
       </c>
       <c r="P219" t="n">
         <v>3</v>
       </c>
       <c r="Q219" t="n">
-        <v>0.0302</v>
+        <v>0.0391</v>
       </c>
       <c r="R219" t="n">
         <v>0.437</v>
@@ -15648,7 +15648,7 @@
         </is>
       </c>
       <c r="K224" t="n">
-        <v>6.6</v>
+        <v>6.1</v>
       </c>
       <c r="L224" t="n">
         <v>2.14</v>
@@ -15660,13 +15660,13 @@
         <v>10</v>
       </c>
       <c r="O224" t="n">
-        <v>6.228999999999999</v>
+        <v>6.079</v>
       </c>
       <c r="P224" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q224" t="n">
-        <v>0.392</v>
+        <v>0.448</v>
       </c>
       <c r="R224" t="n">
         <v>2.915</v>
@@ -15716,7 +15716,7 @@
         </is>
       </c>
       <c r="K225" t="n">
-        <v>7.62</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="L225" t="n">
         <v>2.14</v>
@@ -15728,13 +15728,13 @@
         <v>8.23</v>
       </c>
       <c r="O225" t="n">
-        <v>6.0495</v>
+        <v>6.277500000000001</v>
       </c>
       <c r="P225" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q225" t="n">
-        <v>0.28</v>
+        <v>0.196</v>
       </c>
       <c r="R225" t="n">
         <v>2.915</v>
@@ -15784,7 +15784,7 @@
         </is>
       </c>
       <c r="K226" t="n">
-        <v>7.62</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="L226" t="n">
         <v>2.14</v>
@@ -15796,13 +15796,13 @@
         <v>4.31</v>
       </c>
       <c r="O226" t="n">
-        <v>4.5595</v>
+        <v>4.7875</v>
       </c>
       <c r="P226" t="n">
         <v>3</v>
       </c>
       <c r="Q226" t="n">
-        <v>0.28</v>
+        <v>0.196</v>
       </c>
       <c r="R226" t="n">
         <v>2.915</v>
@@ -15852,7 +15852,7 @@
         </is>
       </c>
       <c r="K227" t="n">
-        <v>8.58</v>
+        <v>8.52</v>
       </c>
       <c r="L227" t="n">
         <v>7.5</v>
@@ -15864,13 +15864,13 @@
         <v>10</v>
       </c>
       <c r="O227" t="n">
-        <v>8.699</v>
+        <v>8.680999999999999</v>
       </c>
       <c r="P227" t="n">
         <v>1</v>
       </c>
       <c r="Q227" t="n">
-        <v>0.1733</v>
+        <v>0.1806</v>
       </c>
       <c r="R227" t="n">
         <v>1.093</v>
@@ -15920,7 +15920,7 @@
         </is>
       </c>
       <c r="K228" t="n">
-        <v>9.52</v>
+        <v>9.32</v>
       </c>
       <c r="L228" t="n">
         <v>7.5</v>
@@ -15932,13 +15932,13 @@
         <v>5.81</v>
       </c>
       <c r="O228" t="n">
-        <v>7.7705</v>
+        <v>7.7105</v>
       </c>
       <c r="P228" t="n">
         <v>2</v>
       </c>
       <c r="Q228" t="n">
-        <v>0.0704</v>
+        <v>0.0924</v>
       </c>
       <c r="R228" t="n">
         <v>1.093</v>
@@ -15988,7 +15988,7 @@
         </is>
       </c>
       <c r="K229" t="n">
-        <v>9.52</v>
+        <v>9.32</v>
       </c>
       <c r="L229" t="n">
         <v>7.7</v>
@@ -16000,13 +16000,13 @@
         <v>3.44</v>
       </c>
       <c r="O229" t="n">
-        <v>7.301</v>
+        <v>7.241</v>
       </c>
       <c r="P229" t="n">
         <v>3</v>
       </c>
       <c r="Q229" t="n">
-        <v>0.0704</v>
+        <v>0.0924</v>
       </c>
       <c r="R229" t="n">
         <v>1.025</v>
@@ -16328,7 +16328,7 @@
         </is>
       </c>
       <c r="K234" t="n">
-        <v>7.48</v>
+        <v>6.7</v>
       </c>
       <c r="L234" t="n">
         <v>0</v>
@@ -16340,13 +16340,13 @@
         <v>4.86</v>
       </c>
       <c r="O234" t="n">
-        <v>4.231</v>
+        <v>3.997</v>
       </c>
       <c r="P234" t="n">
         <v>2</v>
       </c>
       <c r="Q234" t="n">
-        <v>0.2952</v>
+        <v>0.3813</v>
       </c>
       <c r="R234" t="n">
         <v>4.268</v>
@@ -16396,7 +16396,7 @@
         </is>
       </c>
       <c r="K235" t="n">
-        <v>7.48</v>
+        <v>6.7</v>
       </c>
       <c r="L235" t="n">
         <v>0</v>
@@ -16408,13 +16408,13 @@
         <v>1.51</v>
       </c>
       <c r="O235" t="n">
-        <v>2.7185</v>
+        <v>2.4845</v>
       </c>
       <c r="P235" t="n">
         <v>3</v>
       </c>
       <c r="Q235" t="n">
-        <v>0.2952</v>
+        <v>0.3813</v>
       </c>
       <c r="R235" t="n">
         <v>4.002</v>
@@ -16464,7 +16464,7 @@
         </is>
       </c>
       <c r="K236" t="n">
-        <v>9.08</v>
+        <v>8.93</v>
       </c>
       <c r="L236" t="n">
         <v>8.119999999999999</v>
@@ -16476,13 +16476,13 @@
         <v>10</v>
       </c>
       <c r="O236" t="n">
-        <v>9.065999999999999</v>
+        <v>9.020999999999999</v>
       </c>
       <c r="P236" t="n">
         <v>1</v>
       </c>
       <c r="Q236" t="n">
-        <v>0.119</v>
+        <v>0.136</v>
       </c>
       <c r="R236" t="n">
         <v>0.885</v>
@@ -16532,7 +16532,7 @@
         </is>
       </c>
       <c r="K237" t="n">
-        <v>9.380000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="L237" t="n">
         <v>8.279999999999999</v>
@@ -16544,13 +16544,13 @@
         <v>5.19</v>
       </c>
       <c r="O237" t="n">
-        <v>7.412500000000001</v>
+        <v>7.4845</v>
       </c>
       <c r="P237" t="n">
         <v>2</v>
       </c>
       <c r="Q237" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.0595</v>
       </c>
       <c r="R237" t="n">
         <v>0.83</v>
@@ -16600,7 +16600,7 @@
         </is>
       </c>
       <c r="K238" t="n">
-        <v>9.380000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="L238" t="n">
         <v>8.279999999999999</v>
@@ -16612,13 +16612,13 @@
         <v>3.93</v>
       </c>
       <c r="O238" t="n">
-        <v>6.7175</v>
+        <v>6.789499999999999</v>
       </c>
       <c r="P238" t="n">
         <v>3</v>
       </c>
       <c r="Q238" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.0595</v>
       </c>
       <c r="R238" t="n">
         <v>0.83</v>
@@ -16668,7 +16668,7 @@
         </is>
       </c>
       <c r="K239" t="n">
-        <v>8.25</v>
+        <v>8.83</v>
       </c>
       <c r="L239" t="n">
         <v>4.29</v>
@@ -16680,13 +16680,13 @@
         <v>10</v>
       </c>
       <c r="O239" t="n">
-        <v>7.4765</v>
+        <v>7.6505</v>
       </c>
       <c r="P239" t="n">
         <v>1</v>
       </c>
       <c r="Q239" t="n">
-        <v>0.21</v>
+        <v>0.147</v>
       </c>
       <c r="R239" t="n">
         <v>2.186</v>
@@ -16736,7 +16736,7 @@
         </is>
       </c>
       <c r="K240" t="n">
-        <v>7.49</v>
+        <v>7.11</v>
       </c>
       <c r="L240" t="n">
         <v>4.29</v>
@@ -16748,13 +16748,13 @@
         <v>6.91</v>
       </c>
       <c r="O240" t="n">
-        <v>6.389</v>
+        <v>6.275</v>
       </c>
       <c r="P240" t="n">
         <v>2</v>
       </c>
       <c r="Q240" t="n">
-        <v>0.294</v>
+        <v>0.336</v>
       </c>
       <c r="R240" t="n">
         <v>2.186</v>
@@ -16804,7 +16804,7 @@
         </is>
       </c>
       <c r="K241" t="n">
-        <v>8.25</v>
+        <v>8.83</v>
       </c>
       <c r="L241" t="n">
         <v>4.69</v>
@@ -16816,13 +16816,13 @@
         <v>1.71</v>
       </c>
       <c r="O241" t="n">
-        <v>5.329000000000001</v>
+        <v>5.503</v>
       </c>
       <c r="P241" t="n">
         <v>3</v>
       </c>
       <c r="Q241" t="n">
-        <v>0.21</v>
+        <v>0.147</v>
       </c>
       <c r="R241" t="n">
         <v>2.05</v>
@@ -16940,7 +16940,7 @@
         </is>
       </c>
       <c r="K243" t="n">
-        <v>9.359999999999999</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="L243" t="n">
         <v>7.42</v>
@@ -16952,7 +16952,7 @@
         <v>5.19</v>
       </c>
       <c r="O243" t="n">
-        <v>7.669499999999999</v>
+        <v>7.672499999999999</v>
       </c>
       <c r="P243" t="n">
         <v>2</v>
@@ -17008,7 +17008,7 @@
         </is>
       </c>
       <c r="K244" t="n">
-        <v>9.359999999999999</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="L244" t="n">
         <v>7.2</v>
@@ -17020,7 +17020,7 @@
         <v>4.78</v>
       </c>
       <c r="O244" t="n">
-        <v>7.302999999999999</v>
+        <v>7.305999999999999</v>
       </c>
       <c r="P244" t="n">
         <v>3</v>
@@ -17076,7 +17076,7 @@
         </is>
       </c>
       <c r="K245" t="n">
-        <v>9.93</v>
+        <v>9.94</v>
       </c>
       <c r="L245" t="n">
         <v>9.74</v>
@@ -17088,7 +17088,7 @@
         <v>10</v>
       </c>
       <c r="O245" t="n">
-        <v>9.888</v>
+        <v>9.891</v>
       </c>
       <c r="P245" t="n">
         <v>1</v>
@@ -17212,7 +17212,7 @@
         </is>
       </c>
       <c r="K247" t="n">
-        <v>9.93</v>
+        <v>9.94</v>
       </c>
       <c r="L247" t="n">
         <v>9.800000000000001</v>
@@ -17224,7 +17224,7 @@
         <v>2.7</v>
       </c>
       <c r="O247" t="n">
-        <v>7.23</v>
+        <v>7.233000000000001</v>
       </c>
       <c r="P247" t="n">
         <v>3</v>
@@ -17484,7 +17484,7 @@
         </is>
       </c>
       <c r="K251" t="n">
-        <v>6.67</v>
+        <v>6.68</v>
       </c>
       <c r="L251" t="n">
         <v>7.04</v>
@@ -17496,7 +17496,7 @@
         <v>10</v>
       </c>
       <c r="O251" t="n">
-        <v>7.965</v>
+        <v>7.968</v>
       </c>
       <c r="P251" t="n">
         <v>1</v>
@@ -17688,7 +17688,7 @@
         </is>
       </c>
       <c r="K254" t="n">
-        <v>9.77</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="L254" t="n">
         <v>9.43</v>
@@ -17700,13 +17700,13 @@
         <v>10</v>
       </c>
       <c r="O254" t="n">
-        <v>9.731499999999999</v>
+        <v>9.7675</v>
       </c>
       <c r="P254" t="n">
         <v>1</v>
       </c>
       <c r="Q254" t="n">
-        <v>0.042</v>
+        <v>0.0294</v>
       </c>
       <c r="R254" t="n">
         <v>0.437</v>
@@ -17756,7 +17756,7 @@
         </is>
       </c>
       <c r="K255" t="n">
-        <v>9.77</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="L255" t="n">
         <v>9.51</v>
@@ -17768,13 +17768,13 @@
         <v>5.81</v>
       </c>
       <c r="O255" t="n">
-        <v>8.294999999999998</v>
+        <v>8.331</v>
       </c>
       <c r="P255" t="n">
         <v>2</v>
       </c>
       <c r="Q255" t="n">
-        <v>0.042</v>
+        <v>0.0294</v>
       </c>
       <c r="R255" t="n">
         <v>0.41</v>
@@ -17824,7 +17824,7 @@
         </is>
       </c>
       <c r="K256" t="n">
-        <v>9.77</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="L256" t="n">
         <v>9.43</v>
@@ -17836,13 +17836,13 @@
         <v>2.95</v>
       </c>
       <c r="O256" t="n">
-        <v>7.615999999999999</v>
+        <v>7.652</v>
       </c>
       <c r="P256" t="n">
         <v>3</v>
       </c>
       <c r="Q256" t="n">
-        <v>0.042</v>
+        <v>0.0294</v>
       </c>
       <c r="R256" t="n">
         <v>0.437</v>
@@ -18300,7 +18300,7 @@
         </is>
       </c>
       <c r="K263" t="n">
-        <v>9.91</v>
+        <v>9.92</v>
       </c>
       <c r="L263" t="n">
         <v>9.65</v>
@@ -18312,7 +18312,7 @@
         <v>10</v>
       </c>
       <c r="O263" t="n">
-        <v>9.8505</v>
+        <v>9.8535</v>
       </c>
       <c r="P263" t="n">
         <v>1</v>
@@ -18368,7 +18368,7 @@
         </is>
       </c>
       <c r="K264" t="n">
-        <v>9.91</v>
+        <v>9.92</v>
       </c>
       <c r="L264" t="n">
         <v>9.710000000000001</v>
@@ -18380,7 +18380,7 @@
         <v>5.71</v>
       </c>
       <c r="O264" t="n">
-        <v>8.254</v>
+        <v>8.257</v>
       </c>
       <c r="P264" t="n">
         <v>2</v>
@@ -18436,7 +18436,7 @@
         </is>
       </c>
       <c r="K265" t="n">
-        <v>9.91</v>
+        <v>9.92</v>
       </c>
       <c r="L265" t="n">
         <v>9.65</v>
@@ -18448,7 +18448,7 @@
         <v>4.36</v>
       </c>
       <c r="O265" t="n">
-        <v>8.188500000000001</v>
+        <v>8.191500000000001</v>
       </c>
       <c r="P265" t="n">
         <v>3</v>
@@ -18708,7 +18708,7 @@
         </is>
       </c>
       <c r="K269" t="n">
-        <v>9.02</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="L269" t="n">
         <v>6.89</v>
@@ -18720,13 +18720,13 @@
         <v>10</v>
       </c>
       <c r="O269" t="n">
-        <v>8.6175</v>
+        <v>8.7225</v>
       </c>
       <c r="P269" t="n">
         <v>1</v>
       </c>
       <c r="Q269" t="n">
-        <v>0.125</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="R269" t="n">
         <v>1.301</v>
@@ -18776,7 +18776,7 @@
         </is>
       </c>
       <c r="K270" t="n">
-        <v>8.57</v>
+        <v>8.34</v>
       </c>
       <c r="L270" t="n">
         <v>6.89</v>
@@ -18788,13 +18788,13 @@
         <v>5.81</v>
       </c>
       <c r="O270" t="n">
-        <v>7.272</v>
+        <v>7.202999999999999</v>
       </c>
       <c r="P270" t="n">
         <v>2</v>
       </c>
       <c r="Q270" t="n">
-        <v>0.175</v>
+        <v>0.2</v>
       </c>
       <c r="R270" t="n">
         <v>1.301</v>
@@ -18844,7 +18844,7 @@
         </is>
       </c>
       <c r="K271" t="n">
-        <v>9.02</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="L271" t="n">
         <v>6.89</v>
@@ -18856,13 +18856,13 @@
         <v>2.31</v>
       </c>
       <c r="O271" t="n">
-        <v>6.515999999999999</v>
+        <v>6.621</v>
       </c>
       <c r="P271" t="n">
         <v>3</v>
       </c>
       <c r="Q271" t="n">
-        <v>0.125</v>
+        <v>0.08749999999999999</v>
       </c>
       <c r="R271" t="n">
         <v>1.301</v>
@@ -18912,7 +18912,7 @@
         </is>
       </c>
       <c r="K272" t="n">
-        <v>9.619999999999999</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="L272" t="n">
         <v>9.43</v>
@@ -18924,13 +18924,13 @@
         <v>10</v>
       </c>
       <c r="O272" t="n">
-        <v>9.686499999999999</v>
+        <v>9.6655</v>
       </c>
       <c r="P272" t="n">
         <v>1</v>
       </c>
       <c r="Q272" t="n">
-        <v>0.0588</v>
+        <v>0.0672</v>
       </c>
       <c r="R272" t="n">
         <v>0.437</v>
@@ -18980,7 +18980,7 @@
         </is>
       </c>
       <c r="K273" t="n">
-        <v>9.77</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="L273" t="n">
         <v>9.43</v>
@@ -18992,13 +18992,13 @@
         <v>6.21</v>
       </c>
       <c r="O273" t="n">
-        <v>8.648999999999999</v>
+        <v>8.685</v>
       </c>
       <c r="P273" t="n">
         <v>2</v>
       </c>
       <c r="Q273" t="n">
-        <v>0.042</v>
+        <v>0.0294</v>
       </c>
       <c r="R273" t="n">
         <v>0.437</v>
@@ -19048,7 +19048,7 @@
         </is>
       </c>
       <c r="K274" t="n">
-        <v>9.77</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="L274" t="n">
         <v>9.51</v>
@@ -19060,13 +19060,13 @@
         <v>1.51</v>
       </c>
       <c r="O274" t="n">
-        <v>7.057999999999999</v>
+        <v>7.093999999999999</v>
       </c>
       <c r="P274" t="n">
         <v>3</v>
       </c>
       <c r="Q274" t="n">
-        <v>0.042</v>
+        <v>0.0294</v>
       </c>
       <c r="R274" t="n">
         <v>0.41</v>
@@ -19116,7 +19116,7 @@
         </is>
       </c>
       <c r="K275" t="n">
-        <v>7.34</v>
+        <v>8.19</v>
       </c>
       <c r="L275" t="n">
         <v>1.23</v>
@@ -19128,13 +19128,13 @@
         <v>10</v>
       </c>
       <c r="O275" t="n">
-        <v>6.1325</v>
+        <v>6.387499999999999</v>
       </c>
       <c r="P275" t="n">
         <v>1</v>
       </c>
       <c r="Q275" t="n">
-        <v>0.31</v>
+        <v>0.217</v>
       </c>
       <c r="R275" t="n">
         <v>3.227</v>
@@ -19184,7 +19184,7 @@
         </is>
       </c>
       <c r="K276" t="n">
-        <v>7.34</v>
+        <v>8.19</v>
       </c>
       <c r="L276" t="n">
         <v>1.82</v>
@@ -19196,13 +19196,13 @@
         <v>5.67</v>
       </c>
       <c r="O276" t="n">
-        <v>4.827500000000001</v>
+        <v>5.0825</v>
       </c>
       <c r="P276" t="n">
         <v>2</v>
       </c>
       <c r="Q276" t="n">
-        <v>0.31</v>
+        <v>0.217</v>
       </c>
       <c r="R276" t="n">
         <v>3.026</v>
@@ -19252,7 +19252,7 @@
         </is>
       </c>
       <c r="K277" t="n">
-        <v>7.34</v>
+        <v>8.19</v>
       </c>
       <c r="L277" t="n">
         <v>1.23</v>
@@ -19264,13 +19264,13 @@
         <v>2.95</v>
       </c>
       <c r="O277" t="n">
-        <v>4.017</v>
+        <v>4.272</v>
       </c>
       <c r="P277" t="n">
         <v>3</v>
       </c>
       <c r="Q277" t="n">
-        <v>0.31</v>
+        <v>0.217</v>
       </c>
       <c r="R277" t="n">
         <v>3.227</v>
@@ -19524,7 +19524,7 @@
         </is>
       </c>
       <c r="K281" t="n">
-        <v>9.279999999999999</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="L281" t="n">
         <v>9.800000000000001</v>
@@ -19536,7 +19536,7 @@
         <v>10</v>
       </c>
       <c r="O281" t="n">
-        <v>9.714</v>
+        <v>9.716999999999999</v>
       </c>
       <c r="P281" t="n">
         <v>1</v>
@@ -19728,7 +19728,7 @@
         </is>
       </c>
       <c r="K284" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L284" t="n">
         <v>2.14</v>
@@ -19740,7 +19740,7 @@
         <v>10</v>
       </c>
       <c r="O284" t="n">
-        <v>6.715</v>
+        <v>6.718</v>
       </c>
       <c r="P284" t="n">
         <v>1</v>
@@ -19796,7 +19796,7 @@
         </is>
       </c>
       <c r="K285" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L285" t="n">
         <v>2.68</v>
@@ -19808,7 +19808,7 @@
         <v>6.21</v>
       </c>
       <c r="O285" t="n">
-        <v>5.5755</v>
+        <v>5.5785</v>
       </c>
       <c r="P285" t="n">
         <v>2</v>
@@ -19864,7 +19864,7 @@
         </is>
       </c>
       <c r="K286" t="n">
-        <v>8.220000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="L286" t="n">
         <v>2.14</v>
@@ -19876,7 +19876,7 @@
         <v>3.93</v>
       </c>
       <c r="O286" t="n">
-        <v>4.910500000000001</v>
+        <v>4.9135</v>
       </c>
       <c r="P286" t="n">
         <v>3</v>
@@ -19932,7 +19932,7 @@
         </is>
       </c>
       <c r="K287" t="n">
-        <v>9.16</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L287" t="n">
         <v>7.35</v>
@@ -19944,13 +19944,13 @@
         <v>10</v>
       </c>
       <c r="O287" t="n">
-        <v>8.820499999999999</v>
+        <v>8.910499999999999</v>
       </c>
       <c r="P287" t="n">
         <v>1</v>
       </c>
       <c r="Q287" t="n">
-        <v>0.11</v>
+        <v>0.077</v>
       </c>
       <c r="R287" t="n">
         <v>1.145</v>
@@ -20000,7 +20000,7 @@
         </is>
       </c>
       <c r="K288" t="n">
-        <v>8.76</v>
+        <v>8.56</v>
       </c>
       <c r="L288" t="n">
         <v>7.35</v>
@@ -20012,13 +20012,13 @@
         <v>7.15</v>
       </c>
       <c r="O288" t="n">
-        <v>7.919</v>
+        <v>7.858999999999999</v>
       </c>
       <c r="P288" t="n">
         <v>2</v>
       </c>
       <c r="Q288" t="n">
-        <v>0.154</v>
+        <v>0.176</v>
       </c>
       <c r="R288" t="n">
         <v>1.145</v>
@@ -20068,7 +20068,7 @@
         </is>
       </c>
       <c r="K289" t="n">
-        <v>9.16</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="L289" t="n">
         <v>7.35</v>
@@ -20080,13 +20080,13 @@
         <v>2.7</v>
       </c>
       <c r="O289" t="n">
-        <v>6.831499999999999</v>
+        <v>6.9215</v>
       </c>
       <c r="P289" t="n">
         <v>3</v>
       </c>
       <c r="Q289" t="n">
-        <v>0.11</v>
+        <v>0.077</v>
       </c>
       <c r="R289" t="n">
         <v>1.145</v>
@@ -20136,7 +20136,7 @@
         </is>
       </c>
       <c r="K290" t="n">
-        <v>6.91</v>
+        <v>6.92</v>
       </c>
       <c r="L290" t="n">
         <v>2.76</v>
@@ -20148,7 +20148,7 @@
         <v>10</v>
       </c>
       <c r="O290" t="n">
-        <v>6.539</v>
+        <v>6.542</v>
       </c>
       <c r="P290" t="n">
         <v>1</v>
@@ -20204,7 +20204,7 @@
         </is>
       </c>
       <c r="K291" t="n">
-        <v>6.91</v>
+        <v>6.92</v>
       </c>
       <c r="L291" t="n">
         <v>2.76</v>
@@ -20216,7 +20216,7 @@
         <v>6.04</v>
       </c>
       <c r="O291" t="n">
-        <v>5.403</v>
+        <v>5.406</v>
       </c>
       <c r="P291" t="n">
         <v>2</v>
@@ -20272,7 +20272,7 @@
         </is>
       </c>
       <c r="K292" t="n">
-        <v>6.91</v>
+        <v>6.92</v>
       </c>
       <c r="L292" t="n">
         <v>2.76</v>
@@ -20284,7 +20284,7 @@
         <v>3.11</v>
       </c>
       <c r="O292" t="n">
-        <v>4.1775</v>
+        <v>4.1805</v>
       </c>
       <c r="P292" t="n">
         <v>3</v>
@@ -20340,7 +20340,7 @@
         </is>
       </c>
       <c r="K293" t="n">
-        <v>8.609999999999999</v>
+        <v>9.08</v>
       </c>
       <c r="L293" t="n">
         <v>5.51</v>
@@ -20352,13 +20352,13 @@
         <v>10</v>
       </c>
       <c r="O293" t="n">
-        <v>8.0115</v>
+        <v>8.1525</v>
       </c>
       <c r="P293" t="n">
         <v>1</v>
       </c>
       <c r="Q293" t="n">
-        <v>0.17</v>
+        <v>0.119</v>
       </c>
       <c r="R293" t="n">
         <v>1.77</v>
@@ -20408,7 +20408,7 @@
         </is>
       </c>
       <c r="K294" t="n">
-        <v>8.609999999999999</v>
+        <v>9.08</v>
       </c>
       <c r="L294" t="n">
         <v>5.51</v>
@@ -20420,13 +20420,13 @@
         <v>4.64</v>
       </c>
       <c r="O294" t="n">
-        <v>6.249499999999999</v>
+        <v>6.390499999999999</v>
       </c>
       <c r="P294" t="n">
         <v>3</v>
       </c>
       <c r="Q294" t="n">
-        <v>0.17</v>
+        <v>0.119</v>
       </c>
       <c r="R294" t="n">
         <v>1.77</v>
@@ -20476,7 +20476,7 @@
         </is>
       </c>
       <c r="K295" t="n">
-        <v>8.609999999999999</v>
+        <v>9.08</v>
       </c>
       <c r="L295" t="n">
         <v>5.51</v>
@@ -20488,13 +20488,13 @@
         <v>5.71</v>
       </c>
       <c r="O295" t="n">
-        <v>6.933999999999999</v>
+        <v>7.074999999999999</v>
       </c>
       <c r="P295" t="n">
         <v>2</v>
       </c>
       <c r="Q295" t="n">
-        <v>0.17</v>
+        <v>0.119</v>
       </c>
       <c r="R295" t="n">
         <v>1.77</v>
@@ -20544,7 +20544,7 @@
         </is>
       </c>
       <c r="K296" t="n">
-        <v>7.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L296" t="n">
         <v>3.37</v>
@@ -20556,13 +20556,13 @@
         <v>10</v>
       </c>
       <c r="O296" t="n">
-        <v>7.0735</v>
+        <v>7.2685</v>
       </c>
       <c r="P296" t="n">
         <v>1</v>
       </c>
       <c r="Q296" t="n">
-        <v>0.24</v>
+        <v>0.168</v>
       </c>
       <c r="R296" t="n">
         <v>2.498</v>
@@ -20612,7 +20612,7 @@
         </is>
       </c>
       <c r="K297" t="n">
-        <v>7.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L297" t="n">
         <v>3.37</v>
@@ -20624,13 +20624,13 @@
         <v>5.67</v>
       </c>
       <c r="O297" t="n">
-        <v>5.562</v>
+        <v>5.757000000000001</v>
       </c>
       <c r="P297" t="n">
         <v>2</v>
       </c>
       <c r="Q297" t="n">
-        <v>0.24</v>
+        <v>0.168</v>
       </c>
       <c r="R297" t="n">
         <v>2.498</v>
@@ -20680,7 +20680,7 @@
         </is>
       </c>
       <c r="K298" t="n">
-        <v>7.98</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="L298" t="n">
         <v>3.83</v>
@@ -20692,13 +20692,13 @@
         <v>2.47</v>
       </c>
       <c r="O298" t="n">
-        <v>4.353</v>
+        <v>4.548</v>
       </c>
       <c r="P298" t="n">
         <v>3</v>
       </c>
       <c r="Q298" t="n">
-        <v>0.24</v>
+        <v>0.168</v>
       </c>
       <c r="R298" t="n">
         <v>2.342</v>

</xml_diff>